<commit_message>
Double-checking and cleaning up figures and tables
</commit_message>
<xml_diff>
--- a/data/processed/pssi_form_data_altered.xlsx
+++ b/data/processed/pssi_form_data_altered.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\PSSI-final-tech-report\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C44190-B37D-4273-BC40-F836A69EA022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912B8EAF-0CE7-443F-872A-ED495F3C6D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="641">
   <si>
     <t>source_file</t>
   </si>
@@ -391,9 +391,6 @@
     <t>San Juan Chinook</t>
   </si>
   <si>
-    <t>WCVI Fall Chinook</t>
-  </si>
-  <si>
     <t>- San Juan Chinook are a unique population part of the WCVI Fall Chinook CU that has recently received a rebuilding plan. Risk assessments have noted knowledge gaps related to juvenile life stages in the freshwater, estuary and early marine stages. This project aims to fill some of these data gaps.
 - The results from this project will inform a revised risk assessment process for WCVI Chinook in 2026, as well as provide Pacheedaht First Nation with data upon which to base their rebuilding plan for San Juan Chinook and to inform restoration efforts in the watershed.</t>
   </si>
@@ -401,10 +398,6 @@
     <t>These activities will all inform the San Juan Chinook Rebuilding Plan in development by PFN, which will be linked to the broader WCVI Chinook Rebuilding Plan recently developed by DFO (required under the Fish Stock Provisions Act for naturally-produced WCVI Chinook) (DFO 2025). This project will also inform a risk assessment re-scoring expected to happen in 2026, where new information from PSSI projects will be used to re-evaluate the most prominent bottlenecks to WCVI Chinook survival and recovery. The first round WCVI Chinook risk assessment process identified several knowledge gaps, mostly related to early freshwater and marine life cycle stages. For San Juan Chinook specifically, juvenile data from these life stages (and interactions between hatchery and wild juveniles) are sparse, and biological data on natural spawners (e.g., age, origin) are limited.
 These reasons made the San Juan River a good candidate to develop an integrated life history monitoring program in alignment with the larger Follow The Fish program. We focused on activities complemented Pacheedaht First Nation's established juvenile monitoring programs. First, we operated a rotary screw trap program to enumerate and sample naturally-produced out-migrating juveniles (all species, but focused on juvenile Chinook migration timing) in the freshwater environment, allowing us to compare natural migration timing to hatchery release timing, gather baseline biological traits relative to hatchery releases (e.g., size, condition), and estimate fry outmigration abundance. Otolith and stomach samples are also collected from a sub-sample of individuals to assess size-specific survival and diet contents. Second, we collected samples from Pacheedaht's estuary beach seine program to continue examining diet differences and estuary residency (via otolith microchemistry) between hatchery and natural-origin Chinook. Finally, we conducted biweekly purse seining in Port San Juan (PFMA 20-2) through the late spring, summer and fall months (~May-October) to collect mixed-stock information, including hatchery/natural-origin of juvenile Chinook, stock ID, biological traits, relative abundance, and information on other species schooling with Chinook (e.g., Coho, Pacific Herring). As with the RST and beach seine, we also collected otoliths and stomach contents from a sub-sample of Chinook encountered. Finally, we developed a biosampling plan to assess age and stock composition of naturally-spawning adult Chinook (a deadpitch program). Current information on the Proportion of Natural Influence (PNI) is limited only to broodstock sampling, but it is unknown whether these samples are biased and whether they are representative of the river spawning component of the population. It is critical to have an accurate representation of PNI and age and composition-at-return to assess productivity trends and hatchery release strategies for rebuilding San Juan Chinook.
 All work was done in collaboration with Pacheedaht First Nation. Their Fisheries Team lead the majority of the field work and sample collection, as well as advised on sampling designs and salmon dynamics to improve the study design of the project.</t>
-  </si>
-  <si>
-    <t>The key finding of this project will be the specific differences in dynamics between hatchery and natural-origin San Juan Chinook, and using this information to both improve the survival and health of natural-origin juveniles while producing hatchery fish that complement, rather than compete with, the natural population. These findings may be applicable to other systems, although collecting stock-specific information is critical to ensure that any future "indicator" populations are in fact indicative of dynamics in other systems.
-Future studies should further examine specific indicators of early mortality in juvenile salmon, primarily in the freshwater and estuarine stages which are largely unmonitored by DFO. In addition, consideration should be given as to how hatchery release strategies change the life history dynamics of juvenile salmon</t>
   </si>
   <si>
     <t>2404 PSSI Science Project Reporting_Bianucci.docx</t>
@@ -1068,9 +1061,6 @@
   </si>
   <si>
     <t>2425 PSSI Science Project Report - Geospatial Indicators - Jan232026.docx</t>
-  </si>
-  <si>
-    <t>Geospatial Indicators and Metrics for Threats to Fish Habitat in the Fraser River Basin with Thompson-Nicola as a Case Study</t>
   </si>
   <si>
     <t>Josephine Iacarella, Keegan Paterson, Daniel Weller</t>
@@ -2354,39 +2344,6 @@
 CTD PROFILES AND WATER SAMPLING: Profile data were collected using a SeaBird SBE911 CTD with sensors for temperature, salinity, dissolved oxygen, transmissivity (red: 660nm, green: 550 nm) and chlorophyll fluorescence. Water samples were collected using a standard 24-bottle rosette collected on the up-cast. Water samples were analyzed unfiltered for nutrients (nitrate, phosphate, silicate) at the Institute of Ocean Sciences, using a Technicon AutoAnalyzerâ„¢ II (Barwell-Clarke and Whitney, 1996). Nutrient data will be interpreted by calculating molar ratios of Si:N:P and comparing the ratios with those calculated for the Strait of Georgia and Puget Sound. (In Puget Sound, the Si:N ratio has declined since the 1990s, affecting the phytoplankton species assemblage, while the ratio has remained stable in the Strait of Georgia (unpublished data)).
 DATA ARCHIVING: Following quality control, data were archived in the OSD Data Archive at the Institute of Ocean Sciences and made available through the Waterproperties.ca website.
 DELAYS: There were some unforeseen delays in field work and sample analysis. Two sampling cruises were cancelled, and a change in Coast Guard policy that made it impossible to collect sediment cores and water samples during the same cruise, which meant that the field work portion of the project took longer than anticipated. In addition, three labs that had previously analyzed stable isotopes all stopped offering that service, and it took some time to identify a new lab. As a result, some data were only received this month, with the rest of the outstanding data due by March 31. Consequently, only a preliminary interpretation is possible at this time. Interpretation will be completed in the coming fiscal year.</t>
-  </si>
-  <si>
-    <t>â€¢Ahousaht First Nation
-â€¢ Coal Harbour Ltd.
-â€¢ British Columbia Conservation Foundation
-â€¢ Cedar Coast Field Station
-â€¢ Charter Tofino
-â€¢ Ditidaht First Nation
-â€¢ Ehattesaht/Chinehkint First Nation
-â€¢ Ha'oom Fisheries Society
-â€¢ Hesquiaht First Nation
-â€¢ HupaÄasath First Nation
-â€¢ Huu-ay-aht First Nations
-â€¢ The Juanes Lab (University of Victoria)
-â€¢ Ka:'yu:'k't'h'/Che:k:tles7et'h' First Nations
-â€¢ LGL Limited
-â€¢ Maaqutusiis Hahoulthee Stewardship Society
-â€¢ M.C. Wright and Associates Ltd.
-â€¢ Mowachaht-Muchalaht First Nations
-â€¢ Nootka Sound Watershed Society
-â€¢ Nuu-Chah-Nulth Tribal Council
-â€¢ Nuchatlaht Tribe
-â€¢ Pacheedaht First Nation
-â€¢ Pacific Salmon Foundation
-â€¢ Quatsino First Nation
-â€¢ Redd Fish Restoration Society
-â€¢ Thornton Creek Enhancement Society
-â€¢ Tla-o-qui-aht First Nation
-â€¢ Toquaht Nation
-â€¢ Tseshaht First Nation
-â€¢ T'Sou-ke Nation
-â€¢ Uchucklesaht Tribe
-â€¢ YuuÅ‚uÊ”iÅ‚Ê”athÌ£ Government</t>
   </si>
   <si>
     <t>Figure 1. Chinook-bearing river systems on the WCVI that have been genetically sequenced and included in the library for stock assignment with GSI and PBT. Color coding indicates how populations were aggregated for individual stock assignments and shapes indicate how river systems fall in the South-West Vancouver Island (SWVI), Nootka-Kyuquot (NoKy) and North-West Vancouver Island (NWVI) Conservation Units.
@@ -2789,12 +2746,6 @@
 The broodfish-thiamine-injection method appeared to effectively improve the total thiamine levels, mostly in form of TH, in Chinook salmon eggs. Although there were no untreated, control eggs available as a comparison at Shuswap River Hatchery, the injection-treated eggs (20.5 Â± 4.8 nmol/g, range from 16 - 27 nmol/g) contained up to 2 - 3 times the usual thiamine amount in untreated eggs of other Chinook salmon stocks (Figure 2 and 3, 6 - 13 nmol/g). The total thiamine levels in eggs from these injection-treated fish are within the range reported for similar studies on coho salmon (21.925 Â±1.694 nmol/g, Fitzsimons et al., 2005) and steelhead trout *Oncorhynchus mykiss* (total thiamine 20.4 Â± 11.3 nmol/g; Futia et al 2017; mean total thiamine: 33.5 nmol/g, range: 15.4 - 51.1 nmol/g; Reed et al 2023). Unfortunately, our study could not resolve the effectiveness of thiamine bath-treated eggs because of supra-biological and varying levels measured in eggs sampled immediately after the 1 h treatment bath (e.g. 302.5 Â± 31.2 nmol/g in Chinook salmon at Tenderfoot Creek hatchery; 0.95 - 291.20 nmol/g in mid Coho salmon eggs at Capilano Hatchery). Thus, it was unknown how much of the thiamine was actually retained and biologically available to the eggs over time. Future work should resolve the effectiveness and necessity of these thiamine treatments, as these methods could prove highly valuable in both minimizing the potential negative impacts of TDC on early fry and optimizing hatchery salmon production (Futia et al. 2017; Reed et al. 2023; Harder et al. 2025).</t>
   </si>
   <si>
-    <t>Table 1. Results of total thiamine levels detected in chinook salmon eggs treated or untreated with thiamine.
-Figure 1. Results of linear regression analysis on the total mean thiamine level results reported by SUNY Brockport and PSEC on the same set of chinook salmon eggs. Each dot represents an individual sample.
-Figure 2. Results of the total thiamine levels in untreated and unfertilized eggs collected from Capilano mid coho (Cap-mid-Coho, n=5), Chilliwack mid coho (Cwk-mid-Coho, n=10), Tenderfoot Cheakamus Chinook (Tdf-Chinook, n=4), Chilliwack fall Chinook (Cwk-Chinook, n=10), Harrison sockeye (Har-Sockeye, n=10), Chilko sockeye (Cko-Sockeye, n=10), Weaver sockeye (Wvr-Sockeye, n=9) and Chehalis pink (Chs-Pink, n=11). Note that the Harrison sockeye eggs were considered not ripe during sample collection; Tenderfoot Cheakamus Chinook data came from results of untreated eggs reported in Table 1. The dash lines represent thiamine level thresholds established by Mantua et al. (2025) to illustrate the likelihood of being impacted by thiamine deficiency: high - unlikely impacted (&gt; 7.7 nmol/g), intermediate - likely impacted (5.9-7.7 nmol/g), low - impacted (2.7-5.9 nmol/g) and critically low - severely impacted (&lt; 2.7 nmol/g). The cross symbol (Ã—) in the box plot indicates mean values within each group.
-Figure 3. Proportion of salmon eggs from different populations measured by the thiamine level thresholds established by Mantua et al. (2025). Different category of total thiamine level represents different likelihood of being impacted by thiamine deficiency: high - unlikely impacted (&gt; 7.7 nmol/g), intermediate - likely impacted (5.9-7.7 nmol/g), low - impacted (2.7-5.9 nmol/g) and critically low - severely impacted (&lt; 2.7 nmol/g). Eggs were collected from different salmon species and population: Capilano mid coho (n=5), Chilliwack mid coho (n=10), Tenderfoot Cheakamus Chinook (n=4), Chilliwack fall Chinook (n=10), Harrison sockeye (n=10), Chilko sockeye (n=10), Weaver sockeye (n=9) and Chehalis pink (n=11).</t>
-  </si>
-  <si>
     <t>Amcoff, P., BÃ¶rjeson, H., Landergren, P., Vallin, L., and Norrgren, L. 1999. Thiamine (vitamin B1) concentrations in salmon (*Salmo salar*), brown trout (Salmo trutta) and cod (Gadus morhua) from the Baltic Sea. Ambio 28(1): 48-54.
 BÃ¢, A. 2008. Metabolic and structural role of thiamine in nervous tissues. Cell. Mol. Neurobiol. 28(7): 923-931. doi:10.1007/s10571-008-9297-7.
 Brown, S.B., Fitzsimons, J.D., Honeyfield, D.C., and Tillitt, D.E. 2005a. Implications of thiamine deficiency in Great Lakes salmonines. J. Aquat. Anim. Health 17(1): 113-124. doi:10.1577/H04-015.1.
@@ -3219,13 +3170,32 @@
 Figure 2. 2023 daily estimates of Chilko River Sockeye smolt passage: side-looking SONAR estimates versus fence counts.
 Figure 3. 2022 daily estimates of Chilko River Sockeye smolt passage: side-looking SONAR estimates versus fence counts.</t>
   </si>
+  <si>
+    <t>Ahousaht First Nation; Coal Harbour Ltd.; British Columbia Conservation Foundation; Cedar Coast Field Station; Charter Tofino; Ditidaht First Nation; Ehattesaht/Chinehkint First Nation; Ha'oom Fisheries Society; Hesquiaht First Nation; HupaÄasath First Nation; Huu-ay-aht First Nations; The Juanes Lab (University of Victoria); Ka:'yu:'k't'h'/Che:k:tles7et'h' First Nations; LGL Limited; Maaqutusiis Hahoulthee Stewardship Society; M.C. Wright and Associates Ltd.; Mowachaht-Muchalaht First Nations; Nootka Sound Watershed Society; Nuu-Chah-Nulth Tribal Council; Nuchatlaht Tribe; Pacheedaht First Nation; Pacific Salmon Foundation; Quatsino First Nation; Redd Fish Restoration Society; Thornton Creek Enhancement Society; Tla-o-qui-aht First Nation; Toquaht Nation; Tseshaht First Nation; T'Sou-ke Nation; Uchucklesaht Tribe; and YuuÅ‚uÊ”iÅ‚Ê”athÌ£ Government</t>
+  </si>
+  <si>
+    <t>Geospatial indicators and metrics for threats to fish habitat in the Fraser River Basin with Thompson-Nicola as a case study</t>
+  </si>
+  <si>
+    <t>West Coast Vancouver Island Fall Chinook</t>
+  </si>
+  <si>
+    <t>The key finding of this project will be the specific differences in dynamics between hatchery and natural-origin San Juan Chinook, and using this information to both improve the survival and health of natural-origin juveniles while producing hatchery fish that complement, rather than compete with, the natural population. These findings may be applicable to other systems, although collecting stock-specific information is critical to ensure that any future "indicator" populations are in fact indicative of dynamics in other systems.
+Future studies should further examine specific indicators of early mortality in juvenile salmon, primarily in the freshwater and estuarine stages which are largely unmonitored by DFO. In addition, consideration should be given as to how hatchery release strategies change the life history dynamics of juvenile salmon.</t>
+  </si>
+  <si>
+    <t>Table 1. Results of total thiamine levels detected in chinook salmon eggs treated or untreated with thiamine. The results shown were the mean of duplicates. Each test represented results of eggs collected from an individual fish of each population. Note that for Cheakamus chinook salmon, each pair of control and treated eggs (same row) was collected from the same fish. All Middle Shuswap chinook salmon were treated with injection prior to spawning, and thus untreated eggs were not available for sampling. The bath-treated eggs were all fertilized, while the untreated eggs, and the injection-treated eggs were not fertilized. 
+Figure 1. Results of linear regression analysis on the total mean thiamine level results reported by SUNY Brockport and PSEC on the same set of chinook salmon eggs. Each dot represents an individual sample. 
+Figure 2. Results of the total thiamine levels in untreated and unfertilized eggs collected from Capilano mid coho (Cap-mid-Coho, n=5), Chilliwack mid coho (Cwk-mid-Coho, n=10), Tenderfoot Cheakamus Chinook (Tdf-Chinook, n=4), Chilliwack fall Chinook (Cwk-Chinook, n=10), Harrison sockeye (Har-Sockeye, n=10), Chilko sockeye (Cko-Sockeye, n=10), Weaver sockeye (Wvr-Sockeye, n=9) and Chehalis pink (Chs-Pink, n=11). Note that the Harrison sockeye eggs were considered not ripe during sample collection; Tenderfoot Cheakamus Chinook data came from results of untreated eggs reported in Table 1. The dash lines represent thiamine level thresholds established by Mantua et al. (2025) to illustrate the likelihood of being impacted by thiamine deficiency: high - unlikely impacted (&gt; 7.7 nmol/g), intermediate - likely impacted (5.9-7.7 nmol/g), low - impacted (2.7-5.9 nmol/g) and critically low - severely impacted (&lt; 2.7 nmol/g). The cross symbol (Ã—) in the box plot indicates mean values within each group.
+Figure 3. Proportion of salmon eggs from different populations measured by the thiamine level thresholds established by Mantua et al. (2025). Different category of total thiamine level represents different likelihood of being impacted by thiamine deficiency: high - unlikely impacted (&gt; 7.7 nmol/g), intermediate - likely impacted (5.9-7.7 nmol/g), low - impacted (2.7-5.9 nmol/g) and critically low - severely impacted (&lt; 2.7 nmol/g). Eggs were collected from different salmon species and population: Capilano mid coho (n=5), Chilliwack mid coho (n=10), Tenderfoot Cheakamus Chinook (n=4), Chilliwack fall Chinook (n=10), Harrison sockeye (n=10), Chilko sockeye (n=10), Weaver sockeye (n=9) and Chehalis pink (n=11).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -3267,39 +3237,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="23">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3658,6 +3614,24 @@
         <name val="Calibri"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -3696,29 +3670,35 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C1235FC-468F-46C3-9676-E136DE729105}" name="Table1" displayName="Table1" ref="A1:U44" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:U44" xr:uid="{9C1235FC-468F-46C3-9676-E136DE729105}"/>
+  <autoFilter ref="A1:U44" xr:uid="{9C1235FC-468F-46C3-9676-E136DE729105}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="2418"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{21F25E78-D457-418F-9F78-7DE13AE8CD93}" name="source_file" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{B8BCB027-8A7D-4FCE-803F-A296662A280E}" name="extraction_date" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{683393A0-8045-467F-9A16-95D1CB0C532F}" name="project_id" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{5331C13B-A3FC-484A-95E7-7EAD3A2BB00D}" name="project_title" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{65143B71-B457-4DF3-96FB-A320AE4152BD}" name="project_leads" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{0B1052C0-47F1-41AA-B13F-BE70DF38178E}" name="collaborations" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{1204734C-F170-44F7-B4B4-5C53DC28A923}" name="location" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{DB4F19D6-FCB3-4A48-B206-A993711C4060}" name="species" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{3B9CC560-9650-4F10-B6EB-A8BB6D19FD2B}" name="waterbodies" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{3B74A0C4-6035-471F-BA59-5E5296130A6C}" name="life_history" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{83EB77D8-FF38-4BA7-8B8A-C5EB6609BA41}" name="region" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{B5F0F367-295F-4C21-8EF2-8D796262B584}" name="stock" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{592AD976-80C9-41A3-904D-28E27F957093}" name="population" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{0841A155-6170-4816-B52F-62D315F16BB4}" name="cu" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{6A19023B-7495-49F1-A1EC-B098C5E333CF}" name="highlights" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{E075E454-2C61-4348-A20B-0C745E2EC565}" name="background" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{F232593A-A943-4A2F-A957-77EB6182BDA8}" name="methods_findings" dataDxfId="5"/>
-    <tableColumn id="18" xr3:uid="{2F87C396-47EA-4A13-9083-A6C4F71287B3}" name="insights" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{E3203637-205F-4D67-8A5B-15606B06B96D}" name="next_steps" dataDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{71B5C06F-A10D-4B50-AAD8-E218E0D666CD}" name="tables_figures" dataDxfId="2"/>
-    <tableColumn id="21" xr3:uid="{671D065B-E9D7-4645-BF8D-C6523418AA9F}" name="references" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{B8BCB027-8A7D-4FCE-803F-A296662A280E}" name="extraction_date" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{683393A0-8045-467F-9A16-95D1CB0C532F}" name="project_id" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{5331C13B-A3FC-484A-95E7-7EAD3A2BB00D}" name="project_title" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{65143B71-B457-4DF3-96FB-A320AE4152BD}" name="project_leads" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{0B1052C0-47F1-41AA-B13F-BE70DF38178E}" name="collaborations" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{1204734C-F170-44F7-B4B4-5C53DC28A923}" name="location" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{DB4F19D6-FCB3-4A48-B206-A993711C4060}" name="species" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{3B9CC560-9650-4F10-B6EB-A8BB6D19FD2B}" name="waterbodies" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{3B74A0C4-6035-471F-BA59-5E5296130A6C}" name="life_history" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{83EB77D8-FF38-4BA7-8B8A-C5EB6609BA41}" name="region" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{B5F0F367-295F-4C21-8EF2-8D796262B584}" name="stock" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{592AD976-80C9-41A3-904D-28E27F957093}" name="population" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{0841A155-6170-4816-B52F-62D315F16BB4}" name="cu" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{6A19023B-7495-49F1-A1EC-B098C5E333CF}" name="highlights" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{E075E454-2C61-4348-A20B-0C745E2EC565}" name="background" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{F232593A-A943-4A2F-A957-77EB6182BDA8}" name="methods_findings" dataDxfId="4"/>
+    <tableColumn id="18" xr3:uid="{2F87C396-47EA-4A13-9083-A6C4F71287B3}" name="insights" dataDxfId="3"/>
+    <tableColumn id="19" xr3:uid="{E3203637-205F-4D67-8A5B-15606B06B96D}" name="next_steps" dataDxfId="2"/>
+    <tableColumn id="20" xr3:uid="{71B5C06F-A10D-4B50-AAD8-E218E0D666CD}" name="tables_figures" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{671D065B-E9D7-4645-BF8D-C6523418AA9F}" name="references" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4009,7 +3989,7 @@
     <col min="1" max="1" width="13" style="2" customWidth="1"/>
     <col min="2" max="2" width="17.140625" style="6" customWidth="1"/>
     <col min="3" max="3" width="12.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="96.140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" style="2" customWidth="1"/>
     <col min="7" max="8" width="11.42578125" style="2"/>
@@ -4093,7 +4073,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -4134,7 +4114,7 @@
         <v>32</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>33</v>
@@ -4158,7 +4138,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>40</v>
       </c>
@@ -4184,7 +4164,7 @@
         <v>45</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>46</v>
@@ -4193,13 +4173,13 @@
         <v>47</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>48</v>
@@ -4223,7 +4203,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>55</v>
       </c>
@@ -4240,7 +4220,7 @@
         <v>57</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>58</v>
@@ -4249,7 +4229,7 @@
         <v>59</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>60</v>
@@ -4261,19 +4241,19 @@
         <v>61</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>62</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="R4" s="1" t="s">
         <v>63</v>
@@ -4282,13 +4262,13 @@
         <v>64</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>65</v>
       </c>
@@ -4305,10 +4285,10 @@
         <v>67</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>68</v>
@@ -4340,10 +4320,10 @@
         <v>75</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>76</v>
       </c>
@@ -4381,7 +4361,7 @@
         <v>84</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>85</v>
@@ -4393,7 +4373,7 @@
         <v>87</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>88</v>
@@ -4408,74 +4388,74 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:21" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="8">
         <v>46083</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="4">
         <v>2403</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="L7" s="1" t="s">
+      <c r="K7" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="N7" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="O7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="O7" s="1" t="s">
+      <c r="P7" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="P7" s="1" t="s">
+      <c r="Q7" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>639</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="B8" s="7">
         <v>46083</v>
@@ -4484,63 +4464,63 @@
         <v>2404</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="H8" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="J8" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="U8" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="R8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>556</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="B9" s="7">
         <v>46083</v>
@@ -4549,63 +4529,63 @@
         <v>2405</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>68</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O9" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="P9" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="L9" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="R9" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="Q9" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="R9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="U9" s="1" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="B10" s="7">
         <v>46083</v>
@@ -4614,63 +4594,63 @@
         <v>2406</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="H10" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="G10" s="1" t="s">
+      <c r="J10" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I10" s="1" t="s">
+      <c r="L10" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="P10" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="K10" s="1" t="s">
+      <c r="Q10" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="R10" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="L10" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>546</v>
-      </c>
-      <c r="P10" s="1" t="s">
+      <c r="S10" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="Q10" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="R10" s="1" t="s">
+      <c r="T10" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="U10" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="T10" s="1" t="s">
+    </row>
+    <row r="11" spans="1:21" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>135</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>137</v>
       </c>
       <c r="B11" s="8">
         <v>46083</v>
@@ -4679,63 +4659,63 @@
         <v>2407</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>636</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>561</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="I11" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="J11" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>143</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>58</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N11" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="P11" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="Q11" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="P11" s="4" t="s">
+      <c r="R11" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="Q11" s="4" t="s">
+      <c r="S11" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="R11" s="4" t="s">
+      <c r="T11" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="S11" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="T11" s="4" t="s">
-        <v>562</v>
-      </c>
-      <c r="U11" s="4" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="B12" s="7">
         <v>46083</v>
@@ -4744,19 +4724,19 @@
         <v>2408</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>57</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>58</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
@@ -4766,35 +4746,35 @@
         <v>58</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="R12" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="P12" s="1" t="s">
+      <c r="S12" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q12" s="1" t="s">
-        <v>565</v>
-      </c>
-      <c r="R12" s="1" t="s">
+      <c r="T12" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="S12" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="T12" s="1" t="s">
-        <v>566</v>
-      </c>
-      <c r="U12" s="1" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="B13" s="7">
         <v>46083</v>
@@ -4803,61 +4783,61 @@
         <v>2409</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
         <v>68</v>
       </c>
       <c r="I13" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="M13" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N13" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="O13" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="M13" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N13" s="1" t="s">
+      <c r="P13" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="O13" s="1" t="s">
+      <c r="Q13" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="P13" s="1" t="s">
+      <c r="R13" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="Q13" s="1" t="s">
+      <c r="S13" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="R13" s="1" t="s">
+      <c r="T13" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="U13" s="1" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="S13" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>568</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="B14" s="7">
         <v>46083</v>
@@ -4866,22 +4846,22 @@
         <v>2410</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>32</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>32</v>
@@ -4893,36 +4873,36 @@
         <v>32</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>32</v>
       </c>
       <c r="O14" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="P14" s="1" t="s">
+      <c r="R14" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="Q14" s="1" t="s">
+      <c r="S14" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="R14" s="1" t="s">
+      <c r="T14" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="S14" s="1" t="s">
+      <c r="U14" s="1" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>182</v>
       </c>
       <c r="B15" s="7">
         <v>46083</v>
@@ -4931,63 +4911,63 @@
         <v>2412</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="J15" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>58</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="O15" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="S15" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="P15" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="R15" s="1" t="s">
+      <c r="T15" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>191</v>
       </c>
       <c r="B16" s="7">
         <v>46083</v>
@@ -4996,63 +4976,63 @@
         <v>2413</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>576</v>
-      </c>
-      <c r="G16" s="1" t="s">
+      <c r="I16" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="J16" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="I16" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="J16" s="1" t="s">
+      <c r="L16" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O16" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="P16" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="L16" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N16" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O16" s="1" t="s">
+      <c r="Q16" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="P16" s="1" t="s">
+      <c r="R16" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="Q16" s="1" t="s">
+      <c r="S16" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="R16" s="1" t="s">
+      <c r="T16" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="U16" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="S16" s="1" t="s">
+    </row>
+    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>577</v>
-      </c>
-      <c r="U16" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="B17" s="7">
         <v>46083</v>
@@ -5061,63 +5041,63 @@
         <v>2416</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>578</v>
-      </c>
-      <c r="G17" s="1" t="s">
+      <c r="I17" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="K17" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L17" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="M17" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="P17" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="L17" s="1" t="s">
+      <c r="Q17" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="M17" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O17" s="1" t="s">
-        <v>579</v>
-      </c>
-      <c r="P17" s="1" t="s">
+      <c r="R17" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="Q17" s="1" t="s">
+      <c r="S17" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="R17" s="1" t="s">
+      <c r="T17" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="S17" s="1" t="s">
+      <c r="U17" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="T17" s="1" t="s">
+    </row>
+    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>218</v>
       </c>
       <c r="B18" s="7">
         <v>46083</v>
@@ -5126,63 +5106,63 @@
         <v>2417</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="I18" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J18" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="I18" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="M18" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O18" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="P18" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="M18" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O18" s="1" t="s">
+      <c r="Q18" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="S18" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="P18" s="1" t="s">
+      <c r="T18" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>580</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="S18" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>582</v>
-      </c>
-      <c r="U18" s="1" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>230</v>
       </c>
       <c r="B19" s="7">
         <v>46083</v>
@@ -5191,63 +5171,63 @@
         <v>2418</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="F19" s="1" t="s">
+      <c r="I19" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="S19" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="T19" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="U19" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O19" s="1" t="s">
+    </row>
+    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>585</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>586</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="S19" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="T19" s="1" t="s">
-        <v>588</v>
-      </c>
-      <c r="U19" s="1" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>238</v>
       </c>
       <c r="B20" s="7">
         <v>46083</v>
@@ -5256,63 +5236,63 @@
         <v>2421</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>239</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>241</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>58</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="O20" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="P20" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="R20" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="P20" s="1" t="s">
+      <c r="S20" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="Q20" s="1" t="s">
-        <v>591</v>
-      </c>
-      <c r="R20" s="1" t="s">
+      <c r="T20" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="U20" s="1" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="S20" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="T20" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="U20" s="1" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>246</v>
       </c>
       <c r="B21" s="7">
         <v>46083</v>
@@ -5321,63 +5301,63 @@
         <v>2422</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>594</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>595</v>
-      </c>
-      <c r="I21" s="1" t="s">
+      <c r="K21" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L21" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="M21" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O21" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="L21" s="1" t="s">
+      <c r="P21" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="M21" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O21" s="1" t="s">
+      <c r="Q21" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="P21" s="1" t="s">
+      <c r="R21" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="Q21" s="1" t="s">
+      <c r="S21" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="R21" s="1" t="s">
+      <c r="T21" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="S21" s="1" t="s">
+      <c r="U21" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>256</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="U21" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="B22" s="7">
         <v>46083</v>
@@ -5386,63 +5366,63 @@
         <v>2424</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>596</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="H22" s="1" t="s">
+      <c r="J22" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="K22" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="L22" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O22" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="P22" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="R22" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="L22" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O22" s="1" t="s">
+      <c r="S22" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="P22" s="1" t="s">
-        <v>597</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="R22" s="1" t="s">
+      <c r="T22" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="S22" s="1" t="s">
+      <c r="U22" s="1" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="B23" s="7">
         <v>46083</v>
@@ -5450,62 +5430,64 @@
       <c r="C23" s="1">
         <v>2425</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>544</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="I23" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="L23" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N23" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="I23" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="J23" s="1" t="s">
+      <c r="O23" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="P23" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L23" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N23" s="1" t="s">
+      <c r="Q23" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="O23" s="1" t="s">
+      <c r="R23" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="P23" s="1" t="s">
+      <c r="S23" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="Q23" s="1" t="s">
+      <c r="T23" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="U23" s="1" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="R23" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="S23" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>282</v>
       </c>
       <c r="B24" s="7">
         <v>46083</v>
@@ -5514,63 +5496,63 @@
         <v>2426</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>602</v>
-      </c>
-      <c r="G24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="L24" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="M24" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="N24" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="L24" s="1" t="s">
+      <c r="O24" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="M24" s="1" t="s">
+      <c r="P24" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="R24" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="N24" s="1" t="s">
+      <c r="S24" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="O24" s="1" t="s">
+      <c r="T24" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="P24" s="1" t="s">
-        <v>603</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>604</v>
-      </c>
-      <c r="R24" s="1" t="s">
+      <c r="U24" s="1" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="S24" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="U24" s="1" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>297</v>
       </c>
       <c r="B25" s="7">
         <v>46083</v>
@@ -5579,63 +5561,63 @@
         <v>2427</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="K25" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="G25" s="1" t="s">
+      <c r="L25" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O25" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="J25" s="1" t="s">
+      <c r="P25" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="Q25" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="R25" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="L25" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O25" s="1" t="s">
+      <c r="S25" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="P25" s="1" t="s">
+      <c r="T25" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="Q25" s="1" t="s">
-        <v>606</v>
-      </c>
-      <c r="R25" s="1" t="s">
+      <c r="U25" s="1" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="S25" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>307</v>
       </c>
       <c r="B26" s="7">
         <v>46083</v>
@@ -5644,63 +5626,63 @@
         <v>2430</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>608</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="L26" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="M26" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="L26" s="1" t="s">
+      <c r="P26" s="1" t="s">
+        <v>633</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="S26" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="M26" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N26" s="1" t="s">
+      <c r="T26" s="1" t="s">
+        <v>635</v>
+      </c>
+      <c r="U26" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>313</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>638</v>
-      </c>
-      <c r="Q26" s="1" t="s">
-        <v>609</v>
-      </c>
-      <c r="R26" s="1" t="s">
-        <v>639</v>
-      </c>
-      <c r="S26" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="T26" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="U26" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="B27" s="7">
         <v>46083</v>
@@ -5709,63 +5691,63 @@
         <v>2432</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="P27" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>610</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>611</v>
-      </c>
-      <c r="G27" s="1" t="s">
+      <c r="Q27" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M27" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N27" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O27" s="1" t="s">
+      <c r="R27" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="P27" s="1" t="s">
+      <c r="S27" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="Q27" s="1" t="s">
+      <c r="T27" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="R27" s="1" t="s">
+      <c r="U27" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="S27" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="T27" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="U27" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>325</v>
       </c>
       <c r="B28" s="7">
         <v>46083</v>
@@ -5774,63 +5756,63 @@
         <v>2433</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>607</v>
+      </c>
+      <c r="P28" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>610</v>
-      </c>
-      <c r="F28" s="1" t="s">
+      <c r="Q28" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="R28" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N28" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O28" s="1" t="s">
-        <v>612</v>
-      </c>
-      <c r="P28" s="1" t="s">
+      <c r="S28" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="Q28" s="1" t="s">
+      <c r="T28" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="R28" s="1" t="s">
+      <c r="U28" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="S28" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="T28" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="U28" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>334</v>
       </c>
       <c r="B29" s="7">
         <v>46083</v>
@@ -5839,63 +5821,63 @@
         <v>2434</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="G29" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="H29" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I29" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="J29" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="K29" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="L29" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="I29" s="1" t="s">
+      <c r="M29" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="N29" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="L29" s="1" t="s">
+      <c r="O29" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="P29" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="M29" s="1" t="s">
+      <c r="Q29" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="N29" s="1" t="s">
+      <c r="R29" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="O29" s="1" t="s">
-        <v>613</v>
-      </c>
-      <c r="P29" s="1" t="s">
+      <c r="S29" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="Q29" s="1" t="s">
+      <c r="T29" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="R29" s="1" t="s">
+      <c r="U29" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="S29" s="1" t="s">
+    </row>
+    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>347</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="U29" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>350</v>
       </c>
       <c r="B30" s="7">
         <v>46083</v>
@@ -5904,63 +5886,63 @@
         <v>2435</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="K30" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="L30" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="M30" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="N30" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="O30" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="M30" s="1" t="s">
+      <c r="P30" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="N30" s="1" t="s">
+      <c r="Q30" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="O30" s="1" t="s">
+      <c r="R30" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="P30" s="1" t="s">
+      <c r="S30" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="Q30" s="1" t="s">
+      <c r="T30" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="R30" s="1" t="s">
+      <c r="U30" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>365</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="U30" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>368</v>
       </c>
       <c r="B31" s="7">
         <v>46083</v>
@@ -5969,63 +5951,63 @@
         <v>2436</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="G31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="K31" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="L31" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N31" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="O31" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="K31" s="1" t="s">
+      <c r="P31" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="L31" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N31" s="1" t="s">
+      <c r="Q31" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="O31" s="1" t="s">
+      <c r="R31" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="P31" s="1" t="s">
+      <c r="S31" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="Q31" s="1" t="s">
+      <c r="T31" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="R31" s="1" t="s">
+      <c r="U31" s="1" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>380</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="T31" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="U31" s="1" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>383</v>
       </c>
       <c r="B32" s="7">
         <v>46083</v>
@@ -6034,63 +6016,63 @@
         <v>2437</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="I32" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="J32" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="F32" s="1" t="s">
-        <v>615</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="H32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="I32" s="1" t="s">
+      <c r="L32" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="M32" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="N32" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="L32" s="1" t="s">
+      <c r="O32" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="P32" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="M32" s="1" t="s">
+      <c r="Q32" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="N32" s="1" t="s">
+      <c r="R32" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="O32" s="1" t="s">
-        <v>616</v>
-      </c>
-      <c r="P32" s="1" t="s">
+      <c r="S32" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="Q32" s="1" t="s">
+      <c r="T32" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="R32" s="1" t="s">
+      <c r="U32" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="S32" s="1" t="s">
+    </row>
+    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>396</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>399</v>
       </c>
       <c r="B33" s="7">
         <v>46083</v>
@@ -6099,63 +6081,63 @@
         <v>2439</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="H33" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="I33" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="K33" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>617</v>
-      </c>
-      <c r="G33" s="1" t="s">
+      <c r="L33" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="P33" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="Q33" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="K33" s="1" t="s">
+      <c r="R33" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="L33" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O33" s="1" t="s">
+      <c r="S33" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="P33" s="1" t="s">
-        <v>618</v>
-      </c>
-      <c r="Q33" s="1" t="s">
+      <c r="T33" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="R33" s="1" t="s">
+      <c r="U33" s="1" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>407</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="U33" s="1" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>410</v>
       </c>
       <c r="B34" s="7">
         <v>46083</v>
@@ -6164,63 +6146,63 @@
         <v>2442</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="K34" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>620</v>
-      </c>
-      <c r="G34" s="1" t="s">
+      <c r="L34" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="H34" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="I34" s="1" t="s">
+      <c r="M34" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="N34" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="K34" s="1" t="s">
+      <c r="O34" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="L34" s="1" t="s">
+      <c r="P34" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="M34" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="N34" s="1" t="s">
+      <c r="Q34" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="R34" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="O34" s="1" t="s">
+      <c r="S34" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="P34" s="1" t="s">
+      <c r="T34" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="Q34" s="1" t="s">
-        <v>621</v>
-      </c>
-      <c r="R34" s="1" t="s">
+      <c r="U34" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>420</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="U34" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>423</v>
       </c>
       <c r="B35" s="7">
         <v>46083</v>
@@ -6229,63 +6211,63 @@
         <v>2443</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>68</v>
       </c>
       <c r="I35" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="O35" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="P35" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="K35" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N35" s="1" t="s">
+      <c r="Q35" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="O35" s="1" t="s">
+      <c r="R35" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="P35" s="1" t="s">
+      <c r="S35" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="Q35" s="1" t="s">
+      <c r="T35" s="1" t="s">
+        <v>618</v>
+      </c>
+      <c r="U35" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>432</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="T35" s="1" t="s">
-        <v>623</v>
-      </c>
-      <c r="U35" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>435</v>
       </c>
       <c r="B36" s="7">
         <v>46083</v>
@@ -6294,63 +6276,63 @@
         <v>2447</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>81</v>
       </c>
       <c r="I36" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="O36" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="P36" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="K36" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N36" s="1" t="s">
+      <c r="Q36" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="O36" s="1" t="s">
+      <c r="R36" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="P36" s="1" t="s">
+      <c r="S36" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="Q36" s="1" t="s">
+      <c r="T36" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="R36" s="1" t="s">
+      <c r="U36" s="1" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>444</v>
-      </c>
-      <c r="S36" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="T36" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="U36" s="1" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>447</v>
       </c>
       <c r="B37" s="7">
         <v>46083</v>
@@ -6359,63 +6341,63 @@
         <v>2448</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>58</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="I37" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="M37" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="N37" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O37" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="P37" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="L37" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="M37" s="1" t="s">
+      <c r="Q37" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="N37" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O37" s="1" t="s">
+      <c r="R37" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="S37" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="P37" s="1" t="s">
+      <c r="T37" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="Q37" s="1" t="s">
+      <c r="U37" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="R37" s="1" t="s">
-        <v>626</v>
-      </c>
-      <c r="S37" s="1" t="s">
+    </row>
+    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
         <v>458</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="U37" s="1" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>461</v>
       </c>
       <c r="B38" s="7">
         <v>46083</v>
@@ -6424,63 +6406,63 @@
         <v>2449</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="J38" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="K38" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>627</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="H38" s="1" t="s">
+      <c r="L38" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="J38" s="1" t="s">
+      <c r="M38" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="K38" s="1" t="s">
+      <c r="N38" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="L38" s="1" t="s">
+      <c r="O38" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="M38" s="1" t="s">
+      <c r="P38" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="N38" s="1" t="s">
+      <c r="Q38" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="O38" s="1" t="s">
+      <c r="R38" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="P38" s="1" t="s">
+      <c r="S38" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="Q38" s="1" t="s">
+      <c r="T38" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="R38" s="1" t="s">
+      <c r="U38" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="S38" s="1" t="s">
+    </row>
+    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>474</v>
-      </c>
-      <c r="T38" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>477</v>
       </c>
       <c r="B39" s="7">
         <v>46083</v>
@@ -6489,63 +6471,63 @@
         <v>2451</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>81</v>
       </c>
       <c r="I39" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="P39" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="J39" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="L39" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="M39" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="N39" s="1" t="s">
+      <c r="Q39" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="O39" s="1" t="s">
+      <c r="R39" s="1" t="s">
+        <v>623</v>
+      </c>
+      <c r="S39" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="P39" s="1" t="s">
+      <c r="T39" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="Q39" s="1" t="s">
+      <c r="U39" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
         <v>483</v>
-      </c>
-      <c r="R39" s="1" t="s">
-        <v>628</v>
-      </c>
-      <c r="S39" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="T39" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="U39" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>486</v>
       </c>
       <c r="B40" s="7">
         <v>46083</v>
@@ -6554,63 +6536,63 @@
         <v>2452</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="L40" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="I40" s="1" t="s">
+      <c r="M40" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J40" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="K40" s="1" t="s">
+      <c r="N40" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="L40" s="1" t="s">
+      <c r="O40" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="M40" s="1" t="s">
+      <c r="P40" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="N40" s="1" t="s">
+      <c r="Q40" s="1" t="s">
+        <v>624</v>
+      </c>
+      <c r="R40" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="O40" s="1" t="s">
+      <c r="S40" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="P40" s="1" t="s">
+      <c r="T40" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="Q40" s="1" t="s">
-        <v>629</v>
-      </c>
-      <c r="R40" s="1" t="s">
+      <c r="U40" s="1" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
         <v>495</v>
-      </c>
-      <c r="S40" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="T40" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="U40" s="1" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>498</v>
       </c>
       <c r="B41" s="7">
         <v>46083</v>
@@ -6619,63 +6601,63 @@
         <v>2504</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="H41" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>631</v>
-      </c>
-      <c r="G41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="K41" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="L41" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="M41" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="K41" s="1" t="s">
+      <c r="N41" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="O41" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="L41" s="1" t="s">
+      <c r="P41" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="M41" s="1" t="s">
+      <c r="Q41" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="N41" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="O41" s="1" t="s">
+      <c r="R41" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="P41" s="1" t="s">
+      <c r="S41" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="Q41" s="1" t="s">
+      <c r="T41" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="R41" s="1" t="s">
+      <c r="U41" s="1" t="s">
         <v>511</v>
       </c>
-      <c r="S41" s="1" t="s">
+    </row>
+    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
         <v>512</v>
-      </c>
-      <c r="T41" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="U41" s="1" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>515</v>
       </c>
       <c r="B42" s="7">
         <v>46083</v>
@@ -6684,63 +6666,63 @@
         <v>2513</v>
       </c>
       <c r="D42" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L42" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="M42" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="O42" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>632</v>
-      </c>
-      <c r="G42" s="1" t="s">
+      <c r="P42" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="H42" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="L42" s="1" t="s">
+      <c r="Q42" s="1" t="s">
+        <v>628</v>
+      </c>
+      <c r="R42" s="1" t="s">
+        <v>629</v>
+      </c>
+      <c r="S42" s="1" t="s">
         <v>518</v>
       </c>
-      <c r="M42" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="N42" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="O42" s="1" t="s">
+      <c r="T42" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="P42" s="1" t="s">
+      <c r="U42" s="1" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
         <v>520</v>
-      </c>
-      <c r="Q42" s="1" t="s">
-        <v>633</v>
-      </c>
-      <c r="R42" s="1" t="s">
-        <v>634</v>
-      </c>
-      <c r="S42" s="1" t="s">
-        <v>521</v>
-      </c>
-      <c r="T42" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="U42" s="1" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>523</v>
       </c>
       <c r="B43" s="7">
         <v>46083</v>
@@ -6749,22 +6731,22 @@
         <v>2545</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="G43" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="H43" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>526</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>527</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>529</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>32</v>
@@ -6782,30 +6764,30 @@
         <v>32</v>
       </c>
       <c r="O43" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="R43" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="P43" s="1" t="s">
+      <c r="S43" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="Q43" s="1" t="s">
+      <c r="T43" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="R43" s="1" t="s">
+      <c r="U43" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
         <v>533</v>
-      </c>
-      <c r="S43" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="T43" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="U43" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>536</v>
       </c>
       <c r="B44" s="7">
         <v>46083</v>
@@ -6814,13 +6796,13 @@
         <v>3682</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
@@ -6833,25 +6815,25 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
       <c r="O44" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="P44" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="R44" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="P44" s="1" t="s">
+      <c r="S44" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="Q44" s="1" t="s">
+      <c r="T44" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="R44" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="S44" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="T44" s="1" t="s">
-        <v>545</v>
-      </c>
       <c r="U44" s="1" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revising banner and data flow from xlsx to Rmd to Word
</commit_message>
<xml_diff>
--- a/data/processed/pssi_form_data_altered.xlsx
+++ b/data/processed/pssi_form_data_altered.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\PSSI-final-tech-report\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912B8EAF-0CE7-443F-872A-ED495F3C6D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A352C6-1346-4785-B4B8-3962E1484FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,9 +104,6 @@
     <t>0000</t>
   </si>
   <si>
-    <t>Enhanced Mark Selective Fishery (MSF) Monitoring (including a Chinook Reference Fishery)</t>
-  </si>
-  <si>
     <t>Erin Rechisky; Philip Lemp</t>
   </si>
   <si>
@@ -222,9 +219,6 @@
   </si>
   <si>
     <t>2400 PSSI Science Project Reporting_Long_Project.docx</t>
-  </si>
-  <si>
-    <t>Assessment of SEP Chinook and Coho broodstock ELISA screening data by modelling for explanatory variables, and yearling DFAT prevalence data by modelling for predictive variables.</t>
   </si>
   <si>
     <t>Amy Long</t>
@@ -260,9 +254,6 @@
   </si>
   <si>
     <t>2401 PSSI final report-Garver.docx</t>
-  </si>
-  <si>
-    <t>Epidemiological modeling of infectious hematopoietic necrosis virus in Sockeye salmon</t>
   </si>
   <si>
     <t>Kyle Garver</t>
@@ -367,9 +358,6 @@
     <t>2403 PSSI Science Project Reporting - San Juan.docx</t>
   </si>
   <si>
-    <t>San Juan River Adult and Juvenile Assessment Program</t>
-  </si>
-  <si>
     <t>Katie Davidson</t>
   </si>
   <si>
@@ -440,9 +428,6 @@
   </si>
   <si>
     <t>Biological models to support prioritizing salmon stocks under future climates</t>
-  </si>
-  <si>
-    <t>Jan Finke, Travis Tai, Brendan Connors, Cameron Freshwater, Patrick Thompson</t>
   </si>
   <si>
     <t>Amber Holdsworth and Angelica Pena (Ocean Sciences Division); Dan Selbie, Howard Stiff, Greig Oldford, and Josie Iacarella (Ecosystem Science Division)</t>
@@ -580,9 +565,6 @@
   </si>
   <si>
     <t>2408 PSSI Science Project Reporting_Long_Project.docx</t>
-  </si>
-  <si>
-    <t>Improvement, Expansion and Modernization of Salmonid Health Diagnostic Services For Optimizing Salmonid Hatchery Health Management</t>
   </si>
   <si>
     <t>See Supplemental Table 1</t>
@@ -719,9 +701,6 @@
     <t>2412 PSSI Science Project Reporting_Pearce_Mackenzie_Forster_Neville.docx</t>
   </si>
   <si>
-    <t>Investigation of the impacts of singular and coinciding acute climate stressors on the nutritional quality of the pteropod *Limacina helicina*, a juvenile Pacific salmon dietary species</t>
-  </si>
-  <si>
     <t>Chris Pearce, Clara Mackenzie, Ian Forster (DFO, Nearshore Ecosystems Section)</t>
   </si>
   <si>
@@ -1108,11 +1087,6 @@
     <t>2426 PSSI Science Project Reporting Template Oct2025_Sakinaw Sockeye_KP-KF.docx</t>
   </si>
   <si>
-    <t>Sakinaw sockeye juvenile research on measures to increase marine survival
----
-Sakinaw Sockeye Juvenile Research on Measures to Increase Marine Survival</t>
-  </si>
-  <si>
     <t>Kevin Pellett, Karalea Filipovic, Nicolette Watson</t>
   </si>
   <si>
@@ -1362,10 +1336,6 @@
   </si>
   <si>
     <t>2435 PSSI Science Project Reporting - 2453 and 2435.docx</t>
-  </si>
-  <si>
-    <t>Epigenetic variation between hatchery- and natural-origin Canadian Chinook salmon
-intergeneration transfer and parental origins of DNA methylation variation in coho and Chinook salmon (2435 and 2453)</t>
   </si>
   <si>
     <t>Timothy Healy, Kyle Wellband, Eric Rondeau</t>
@@ -1881,9 +1851,6 @@
   </si>
   <si>
     <t>2449 PSSI Science Project Reporting- salmonMSE.docx</t>
-  </si>
-  <si>
-    <t>A decision-support tool that considers harvest, hatchery, and habitat management levers to support implementation of the *Fisheries Act* for Pacific salmon</t>
   </si>
   <si>
     <t>Carrie Holt, Catarina Wor and Brendan Connors</t>
@@ -2847,9 +2814,6 @@
     <t>Chinook Salmon *OncorhynchusÂ tshawytscha*</t>
   </si>
   <si>
-    <t>Doug Braun, Josephine Iacarella, SecwÃ©pemc Fisheries Commission</t>
-  </si>
-  <si>
     <t>Low flows during summer months can be an important bottleneck for stream-rearing rearing salmon. Determining how much water fish need is therefore a critical management question, especially given rising human water use and climate warming. Elevated water temperature is another threat facing stream-rearing salmon that is often linked to low flows. However, conventional modelling tools for determining instream flow needs have generally not explicitly considered temperature. This is a gap for management as it is unclear if current instream flow assessments will apply in a warmer future.
 This project developed an analytical framework to integrate water temperature into habitat simulation models, a widely used tool for determining instream flow needs. We used a bioenergetics framework that relates channel hydraulics (e.g., depth and velocity) and temperature to the daily energy balance of juvenile salmonids. We then applied the approach to 17 coho-rearing streams across the North Thompson watershed, interior BC. This work was collaborative with SecwÃ©pemc Fisheries Commission and Simpcw First Nation and will inform instream flow management through the lens of climate change.</t>
   </si>
@@ -2875,9 +2839,6 @@
 Iacarella, J.C. and Weller, J.D., 2023. Predicting favourable streams for anadromous salmon spawning and natal rearing under climate change.Â Can. J. Fish. Aquat. Sci.,Â 81(1), pp.1-13. doi:10.1139/cjfas-2023-0096
 Iacarella, J.C., Paterson, K., Potapova, A., and Weller, J.D. 2025. Geospatial Indicators and Metrics for Threats to Fish Habitat in the Fraser River Basin with Thompson-Nicola as a Case Study. DFO Can. Sci. Advis. Sec. Res. Doc. 2025/013. xiii + 126 p.
 Rosenfeld, J., Gonzalez-Espinosa, P., Jarvis, L., Enders, E., Bayly, M., Paul, A., MacPherson, L., Moore, J., Sullivan, M., Ulaski, M., and Wilson, K. 2022. Stressor-response functions as a generalizable model for context dependence. Trends Ecol. Evolut. 37: 1032-1035. doi:10.1016/j.tree.2022.09.010</t>
-  </si>
-  <si>
-    <t>shÃ­shÃ¡lh Nation</t>
   </si>
   <si>
     <t>Sakinaw sockeye have been listed as endangered with COSEWIC since 2003, and a *Species at Risk Act* Recovery Potential Assessment (RPA) was completed in 2017 (Ramshaw et al. 2019). The RPA cited low marine survival as the greatest limiting factor in recovery, with predator abundance and assumed predation on smolts and adults ranked as high risk, with a critical level of impact. Perpetually low marine survivals are preventing recovery such that the persistence of the population is entirely dependent on a captive brood program.
@@ -2935,9 +2896,6 @@
 SONAR data was manually reviewed and edited using Echoview software to remove noise, and echo integrated in 1 hour x 1 m range cells (side-looking) or 1 hour x 0.2 m range cells (up-looking). The results were exported as csv files, and all echo integration csv files belonging to the same transducer and site were concatenated for further analysis in Microsoft Excel. Excel was then used to convert the echo integration results to smolt passage estimates, which were then compared to the estimates generated at the Chilko River smolt enumeration fence.
 In 2023 and 2024 (2025 results pending), daily estimates of smolt passage showed close correspondence (5% in 2023, 9% in 2024) between fence counts and independent acoustic estimates both in time and magnitude. In the first year of the study (2022), daily SONAR estimates were in good agreement with the fence counts over the first 9 days of the study, but consistently higher over the last 9 days (May 3rd and thereafter). At present, the source of this divergence is unclear.
 This project is one of few that have used split-beam SONARs configured in this manner to enumerate outmigrating salmon smolts. While further testing needs to be conducted in both the Chilko River where the study was conducted, and in other candidate systems, the preliminary results of this study are promising. These methods could be modified and applied to a variety of salmon stock assessment programs to gain crucial information on survival in the early freshwater life stages (egg to smolt survival), however, considerable planning and care needs to be taken when selecting a suitable site.</t>
-  </si>
-  <si>
-    <t>StÃ©phane Gauthier</t>
   </si>
   <si>
     <t>Follow The fish team</t>
@@ -3171,9 +3129,6 @@
 Figure 3. 2022 daily estimates of Chilko River Sockeye smolt passage: side-looking SONAR estimates versus fence counts.</t>
   </si>
   <si>
-    <t>Ahousaht First Nation; Coal Harbour Ltd.; British Columbia Conservation Foundation; Cedar Coast Field Station; Charter Tofino; Ditidaht First Nation; Ehattesaht/Chinehkint First Nation; Ha'oom Fisheries Society; Hesquiaht First Nation; HupaÄasath First Nation; Huu-ay-aht First Nations; The Juanes Lab (University of Victoria); Ka:'yu:'k't'h'/Che:k:tles7et'h' First Nations; LGL Limited; Maaqutusiis Hahoulthee Stewardship Society; M.C. Wright and Associates Ltd.; Mowachaht-Muchalaht First Nations; Nootka Sound Watershed Society; Nuu-Chah-Nulth Tribal Council; Nuchatlaht Tribe; Pacheedaht First Nation; Pacific Salmon Foundation; Quatsino First Nation; Redd Fish Restoration Society; Thornton Creek Enhancement Society; Tla-o-qui-aht First Nation; Toquaht Nation; Tseshaht First Nation; T'Sou-ke Nation; Uchucklesaht Tribe; and YuuÅ‚uÊ”iÅ‚Ê”athÌ£ Government</t>
-  </si>
-  <si>
     <t>Geospatial indicators and metrics for threats to fish habitat in the Fraser River Basin with Thompson-Nicola as a case study</t>
   </si>
   <si>
@@ -3188,6 +3143,70 @@
 Figure 1. Results of linear regression analysis on the total mean thiamine level results reported by SUNY Brockport and PSEC on the same set of chinook salmon eggs. Each dot represents an individual sample. 
 Figure 2. Results of the total thiamine levels in untreated and unfertilized eggs collected from Capilano mid coho (Cap-mid-Coho, n=5), Chilliwack mid coho (Cwk-mid-Coho, n=10), Tenderfoot Cheakamus Chinook (Tdf-Chinook, n=4), Chilliwack fall Chinook (Cwk-Chinook, n=10), Harrison sockeye (Har-Sockeye, n=10), Chilko sockeye (Cko-Sockeye, n=10), Weaver sockeye (Wvr-Sockeye, n=9) and Chehalis pink (Chs-Pink, n=11). Note that the Harrison sockeye eggs were considered not ripe during sample collection; Tenderfoot Cheakamus Chinook data came from results of untreated eggs reported in Table 1. The dash lines represent thiamine level thresholds established by Mantua et al. (2025) to illustrate the likelihood of being impacted by thiamine deficiency: high - unlikely impacted (&gt; 7.7 nmol/g), intermediate - likely impacted (5.9-7.7 nmol/g), low - impacted (2.7-5.9 nmol/g) and critically low - severely impacted (&lt; 2.7 nmol/g). The cross symbol (Ã—) in the box plot indicates mean values within each group.
 Figure 3. Proportion of salmon eggs from different populations measured by the thiamine level thresholds established by Mantua et al. (2025). Different category of total thiamine level represents different likelihood of being impacted by thiamine deficiency: high - unlikely impacted (&gt; 7.7 nmol/g), intermediate - likely impacted (5.9-7.7 nmol/g), low - impacted (2.7-5.9 nmol/g) and critically low - severely impacted (&lt; 2.7 nmol/g). Eggs were collected from different salmon species and population: Capilano mid coho (n=5), Chilliwack mid coho (n=10), Tenderfoot Cheakamus Chinook (n=4), Chilliwack fall Chinook (n=10), Harrison sockeye (n=10), Chilko sockeye (n=10), Weaver sockeye (n=9) and Chehalis pink (n=11).</t>
+  </si>
+  <si>
+    <t>shíshálh Nation</t>
+  </si>
+  <si>
+    <t>Sakinaw sockeye juvenile research on measures to increase marine survival</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Investigation of the impacts of singular and coinciding acute climate stressors on the nutritional quality of the pteropod </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Limacina helicina</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>, a juvenile Pacific salmon dietary species</t>
+    </r>
+  </si>
+  <si>
+    <t>Epigenetic variation between hatchery- and natural-origin Canadian Chinook salmon intergeneration transfer and parental origins of DNA methylation variation in coho and Chinook salmon (2435 and 2453)</t>
+  </si>
+  <si>
+    <t>A decision-support tool that considers harvest, hatchery, and habitat management levers to support implementation of the Fisheries Act for Pacific salmon</t>
+  </si>
+  <si>
+    <t>Jan Finke, Travis Tai, Brendan Connors, 
+Cameron Freshwater, Patrick Thompson</t>
+  </si>
+  <si>
+    <t>Stéphane Gauthier</t>
+  </si>
+  <si>
+    <t>Ahousaht First Nation; Coal Harbour Ltd.; British Columbia Conservation Foundation; Cedar Coast Field Station; Charter Tofino; Ditidaht First Nation; Ehattesaht/Chinehkint First Nation; Ha’oom Fisheries Society; Hesquiaht First Nation; Hupačasath First Nation; Huu-ay-aht First Nations; The Juanes Lab (University of Victoria); Ka:’yu:’k’t’h’/Che:k:tles7et’h’ First Nations; LGL Limited; Maaqutusiis Hahoulthee Stewardship Society; M.C. Wright and Associates Ltd.; Mowachaht-Muchalaht First Nations; Nootka Sound Watershed Society; Nuu-Chah-Nulth Tribal Council; Nuchatlaht Tribe; Pacheedaht First Nation; Pacific Salmon Foundation; Quatsino First Nation; Redd Fish Restoration Society; Thornton Creek Enhancement Society; Tla-o-qui-aht First Nation; Toquaht Nation; Tseshaht First Nation; T’Sou-ke Nation; Uchucklesaht Tribe; Yuułuʔiłʔatḥ Government</t>
+  </si>
+  <si>
+    <t>Doug Braun, Josephine Iacarella, Secwépemc Fisheries Commission</t>
+  </si>
+  <si>
+    <t>Enhanced Mark Selective Fishery (MSF) monitoring (including a Chinook Reference Fishery)</t>
+  </si>
+  <si>
+    <t>Assessment of SEP Chinook and coho broodstock ELISA screening data by modelling for explanatory variables, and yearling DFAT prevalence data by modelling for predictive variables.</t>
+  </si>
+  <si>
+    <t>Epidemiological modeling of infectious hematopoietic necrosis virus in sockeye salmon</t>
+  </si>
+  <si>
+    <t>San Juan River adult and juvenile assessment program</t>
+  </si>
+  <si>
+    <t>Improvement, expansion and modernization of salmonid health diagnostic services for optimizing salmonid hatchery health management</t>
   </si>
 </sst>
 </file>
@@ -3197,7 +3216,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3211,6 +3230,13 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -3237,7 +3263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3248,9 +3274,6 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3670,13 +3693,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C1235FC-468F-46C3-9676-E136DE729105}" name="Table1" displayName="Table1" ref="A1:U44" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:U44" xr:uid="{9C1235FC-468F-46C3-9676-E136DE729105}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="2418"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:U44" xr:uid="{9C1235FC-468F-46C3-9676-E136DE729105}"/>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{21F25E78-D457-418F-9F78-7DE13AE8CD93}" name="source_file" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{B8BCB027-8A7D-4FCE-803F-A296662A280E}" name="extraction_date" dataDxfId="19"/>
@@ -4073,7 +4090,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -4083,64 +4100,64 @@
       <c r="C2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="9" t="s">
+        <v>636</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="N2" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="U2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="B3" s="7">
         <v>46083</v>
@@ -4149,63 +4166,63 @@
         <v>2394</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O3" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="R3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="T3" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="U3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="U3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="B4" s="7">
         <v>46083</v>
@@ -4213,64 +4230,64 @@
       <c r="C4" s="1">
         <v>2400</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>545</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="I4" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="K4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J4" s="1" t="s">
+      <c r="M4" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="L4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="M4" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>546</v>
-      </c>
-      <c r="P4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="Q4" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="R4" s="1" t="s">
+      <c r="T4" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>548</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="B5" s="7">
         <v>46083</v>
@@ -4278,23 +4295,23 @@
       <c r="C5" s="1">
         <v>2401</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="9" t="s">
+        <v>638</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -4302,30 +4319,30 @@
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="R5" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="T5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="R5" s="1" t="s">
+      <c r="U5" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="B6" s="7">
         <v>46083</v>
@@ -4334,63 +4351,63 @@
         <v>2402</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="K6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="M6" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="L6" s="1" t="s">
+      <c r="P6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="R6" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="T6" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="Q6" s="1" t="s">
-        <v>549</v>
-      </c>
-      <c r="R6" s="1" t="s">
+      <c r="U6" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="S6" s="1" t="s">
+    </row>
+    <row r="7" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="B7" s="8">
         <v>46083</v>
@@ -4398,64 +4415,64 @@
       <c r="C7" s="4">
         <v>2403</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
+        <v>639</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="I7" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="K7" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="M7" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="O7" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="P7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="Q7" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>638</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q7" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="R7" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>639</v>
-      </c>
-      <c r="T7" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="U7" s="4" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="B8" s="7">
         <v>46083</v>
@@ -4464,63 +4481,63 @@
         <v>2404</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="L8" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="G8" s="1" t="s">
+      <c r="P8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="Q8" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="U8" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="I8" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>552</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>553</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="B9" s="7">
         <v>46083</v>
@@ -4529,63 +4546,63 @@
         <v>2405</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>632</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="P9" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="Q9" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="R9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J9" s="1" t="s">
+      <c r="S9" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="L9" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O9" s="1" t="s">
+      <c r="U9" s="1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="B10" s="7">
         <v>46083</v>
@@ -4594,63 +4611,63 @@
         <v>2406</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="P10" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="Q10" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="R10" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="G10" s="1" t="s">
+      <c r="S10" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="I10" s="1" t="s">
+      <c r="T10" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="K10" s="1" t="s">
+      <c r="U10" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="L10" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N10" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="P10" s="1" t="s">
+    </row>
+    <row r="11" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>557</v>
-      </c>
-      <c r="R10" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="B11" s="8">
         <v>46083</v>
@@ -4659,63 +4676,63 @@
         <v>2407</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>634</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="J11" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="K11" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="N11" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>636</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="O11" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="P11" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="Q11" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="R11" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="K11" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="N11" s="4" t="s">
+      <c r="S11" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="T11" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q11" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="R11" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="S11" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="T11" s="4" t="s">
-        <v>558</v>
-      </c>
-      <c r="U11" s="4" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="B12" s="7">
         <v>46083</v>
@@ -4723,58 +4740,58 @@
       <c r="C12" s="1">
         <v>2408</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>149</v>
+      <c r="D12" s="9" t="s">
+        <v>640</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>560</v>
+        <v>550</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>561</v>
+        <v>551</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>562</v>
+        <v>552</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>563</v>
+        <v>553</v>
       </c>
     </row>
-    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B13" s="7">
         <v>46083</v>
@@ -4783,61 +4800,61 @@
         <v>2409</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I13" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="P13" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="Q13" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="R13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="S13" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="M13" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N13" s="1" t="s">
+      <c r="T13" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="U13" s="1" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="Q13" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="R13" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="S13" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="B14" s="7">
         <v>46083</v>
@@ -4846,63 +4863,63 @@
         <v>2410</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="R14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="S14" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>566</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="I14" s="1" t="s">
+      <c r="T14" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M14" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O14" s="1" t="s">
+      <c r="U14" s="1" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q14" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="S14" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="B15" s="7">
         <v>46083</v>
@@ -4910,64 +4927,64 @@
       <c r="C15" s="1">
         <v>2412</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="9" t="s">
+        <v>629</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="S15" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="T15" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>568</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>569</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="B16" s="7">
         <v>46083</v>
@@ -4976,63 +4993,63 @@
         <v>2413</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="P16" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="Q16" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="G16" s="1" t="s">
+      <c r="R16" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="S16" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="I16" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="J16" s="1" t="s">
+      <c r="T16" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="U16" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="K16" s="1" t="s">
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N16" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="S16" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="U16" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="B17" s="7">
         <v>46083</v>
@@ -5041,63 +5058,63 @@
         <v>2416</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="P17" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="Q17" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="G17" s="1" t="s">
+      <c r="R17" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="S17" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="T17" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="U17" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="L17" s="1" t="s">
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O17" s="1" t="s">
-        <v>575</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="R17" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="S17" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="T17" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="B18" s="7">
         <v>46083</v>
@@ -5106,63 +5123,63 @@
         <v>2417</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="L18" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="M18" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O18" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="P18" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="Q18" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="S18" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="T18" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="M18" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>576</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>577</v>
-      </c>
-      <c r="S18" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>578</v>
-      </c>
-      <c r="U18" s="1" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>228</v>
       </c>
       <c r="B19" s="7">
         <v>46083</v>
@@ -5171,63 +5188,63 @@
         <v>2418</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="S19" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="T19" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="U19" s="1" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>580</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O19" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>582</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>583</v>
-      </c>
-      <c r="S19" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="T19" s="10" t="s">
-        <v>640</v>
-      </c>
-      <c r="U19" s="1" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>236</v>
       </c>
       <c r="B20" s="7">
         <v>46083</v>
@@ -5236,63 +5253,63 @@
         <v>2421</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="P20" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="S20" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="T20" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="U20" s="1" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>237</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>585</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N20" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O20" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="Q20" s="1" t="s">
-        <v>586</v>
-      </c>
-      <c r="R20" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="S20" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="T20" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="U20" s="1" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>244</v>
       </c>
       <c r="B21" s="7">
         <v>46083</v>
@@ -5301,63 +5318,63 @@
         <v>2422</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q21" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="R21" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="I21" s="1" t="s">
+      <c r="S21" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="T21" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="L21" s="1" t="s">
+      <c r="U21" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="R21" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="S21" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="U21" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>256</v>
       </c>
       <c r="B22" s="7">
         <v>46083</v>
@@ -5366,63 +5383,63 @@
         <v>2424</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>635</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="R22" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="S22" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>591</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H22" s="1" t="s">
+      <c r="T22" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="U22" s="1" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>593</v>
-      </c>
-      <c r="R22" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="S22" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>267</v>
       </c>
       <c r="B23" s="7">
         <v>46083</v>
@@ -5431,63 +5448,63 @@
         <v>2425</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>637</v>
+        <v>623</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="P23" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="F23" s="9" t="s">
-        <v>544</v>
-      </c>
-      <c r="G23" s="1" t="s">
+      <c r="Q23" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="R23" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="I23" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="J23" s="1" t="s">
+      <c r="S23" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="T23" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="U23" s="1" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="R23" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="S23" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>595</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>279</v>
       </c>
       <c r="B24" s="7">
         <v>46083</v>
@@ -5495,64 +5512,64 @@
       <c r="C24" s="1">
         <v>2426</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="9" t="s">
+        <v>628</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>627</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="M24" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="N24" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>597</v>
-      </c>
-      <c r="G24" s="1" t="s">
+      <c r="O24" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="P24" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="R24" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="S24" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="T24" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="U24" s="1" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>286</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="N24" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="O24" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="P24" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>599</v>
-      </c>
-      <c r="R24" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="S24" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="U24" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>294</v>
       </c>
       <c r="B25" s="7">
         <v>46083</v>
@@ -5561,63 +5578,63 @@
         <v>2427</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="S25" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="T25" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="G25" s="1" t="s">
+      <c r="U25" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>296</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="P25" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="Q25" s="1" t="s">
-        <v>601</v>
-      </c>
-      <c r="R25" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="S25" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="B26" s="7">
         <v>46083</v>
@@ -5626,63 +5643,63 @@
         <v>2430</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>632</v>
+        <v>619</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="S26" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="T26" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="U26" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>305</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>603</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="L26" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>633</v>
-      </c>
-      <c r="Q26" s="1" t="s">
-        <v>604</v>
-      </c>
-      <c r="R26" s="1" t="s">
-        <v>634</v>
-      </c>
-      <c r="S26" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="T26" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="U26" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="B27" s="7">
         <v>46083</v>
@@ -5691,63 +5708,63 @@
         <v>2432</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>633</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="P27" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="Q27" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="S27" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="T27" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="U27" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>314</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>605</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>606</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M27" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N27" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O27" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="P27" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="Q27" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="R27" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="S27" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="T27" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="U27" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>322</v>
       </c>
       <c r="B28" s="7">
         <v>46083</v>
@@ -5756,63 +5773,63 @@
         <v>2433</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>633</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="P28" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="S28" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="T28" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="U28" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>323</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>605</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N28" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O28" s="1" t="s">
-        <v>607</v>
-      </c>
-      <c r="P28" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="Q28" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="R28" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="S28" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="T28" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="U28" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>331</v>
       </c>
       <c r="B29" s="7">
         <v>46083</v>
@@ -5821,63 +5838,63 @@
         <v>2434</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="N29" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="O29" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="P29" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="Q29" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="R29" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="I29" s="1" t="s">
+      <c r="S29" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="T29" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="L29" s="1" t="s">
+      <c r="U29" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="M29" s="1" t="s">
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>339</v>
-      </c>
-      <c r="N29" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="O29" s="1" t="s">
-        <v>608</v>
-      </c>
-      <c r="P29" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="Q29" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="R29" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="S29" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="U29" s="1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>347</v>
       </c>
       <c r="B30" s="7">
         <v>46083</v>
@@ -5885,64 +5902,64 @@
       <c r="C30" s="1">
         <v>2435</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="9" t="s">
+        <v>630</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="M30" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="N30" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="O30" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="P30" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="Q30" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="R30" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="S30" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="T30" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="U30" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>356</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="N30" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>360</v>
-      </c>
-      <c r="Q30" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="R30" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="U30" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>365</v>
       </c>
       <c r="B31" s="7">
         <v>46083</v>
@@ -5951,63 +5968,63 @@
         <v>2436</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="P31" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="Q31" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="G31" s="1" t="s">
+      <c r="R31" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="S31" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="T31" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="U31" s="1" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>371</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>375</v>
-      </c>
-      <c r="Q31" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>377</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="T31" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="U31" s="1" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>380</v>
       </c>
       <c r="B32" s="7">
         <v>46083</v>
@@ -6016,63 +6033,63 @@
         <v>2437</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="P32" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="Q32" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="F32" s="1" t="s">
-        <v>610</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="H32" s="1" t="s">
+      <c r="R32" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="I32" s="1" t="s">
+      <c r="S32" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="T32" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="U32" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="L32" s="1" t="s">
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>387</v>
-      </c>
-      <c r="M32" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="N32" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>611</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>390</v>
-      </c>
-      <c r="Q32" s="1" t="s">
-        <v>391</v>
-      </c>
-      <c r="R32" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>396</v>
       </c>
       <c r="B33" s="7">
         <v>46083</v>
@@ -6081,63 +6098,63 @@
         <v>2439</v>
       </c>
       <c r="D33" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="P33" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="Q33" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="R33" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="S33" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="T33" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="U33" s="1" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>398</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>612</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="P33" s="1" t="s">
-        <v>613</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="R33" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="U33" s="1" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>407</v>
       </c>
       <c r="B34" s="7">
         <v>46083</v>
@@ -6146,63 +6163,63 @@
         <v>2442</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="N34" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="P34" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="Q34" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="R34" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="S34" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>615</v>
-      </c>
-      <c r="G34" s="1" t="s">
+      <c r="T34" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="H34" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="J34" s="1" t="s">
+      <c r="U34" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>411</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="L34" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="M34" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="N34" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="O34" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="P34" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>616</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="U34" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>420</v>
       </c>
       <c r="B35" s="7">
         <v>46083</v>
@@ -6211,63 +6228,63 @@
         <v>2443</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="P35" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="R35" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="S35" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>617</v>
-      </c>
-      <c r="G35" s="1" t="s">
+      <c r="T35" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="U35" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>423</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="T35" s="1" t="s">
-        <v>618</v>
-      </c>
-      <c r="U35" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>432</v>
       </c>
       <c r="B36" s="7">
         <v>46083</v>
@@ -6276,63 +6293,63 @@
         <v>2447</v>
       </c>
       <c r="D36" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="S36" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="T36" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>619</v>
-      </c>
-      <c r="G36" s="1" t="s">
+      <c r="U36" s="1" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>435</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="O36" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="P36" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q36" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="R36" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="S36" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="T36" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="U36" s="1" t="s">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>444</v>
       </c>
       <c r="B37" s="7">
         <v>46083</v>
@@ -6341,63 +6358,63 @@
         <v>2448</v>
       </c>
       <c r="D37" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="P37" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="Q37" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="R37" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="S37" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="T37" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="G37" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="I37" s="1" t="s">
+      <c r="U37" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="J37" s="1" t="s">
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
         <v>449</v>
-      </c>
-      <c r="K37" s="1" t="s">
-        <v>450</v>
-      </c>
-      <c r="L37" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="M37" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="P37" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="Q37" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="R37" s="1" t="s">
-        <v>621</v>
-      </c>
-      <c r="S37" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="U37" s="1" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>458</v>
       </c>
       <c r="B38" s="7">
         <v>46083</v>
@@ -6405,64 +6422,64 @@
       <c r="C38" s="1">
         <v>2449</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="9" t="s">
+        <v>631</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="P38" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="Q38" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="R38" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>622</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="H38" s="1" t="s">
+      <c r="S38" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>544</v>
-      </c>
-      <c r="J38" s="1" t="s">
+      <c r="T38" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="K38" s="1" t="s">
+      <c r="U38" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="L38" s="1" t="s">
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>464</v>
-      </c>
-      <c r="M38" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="N38" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="P38" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="Q38" s="1" t="s">
-        <v>469</v>
-      </c>
-      <c r="R38" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="S38" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="T38" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>474</v>
       </c>
       <c r="B39" s="7">
         <v>46083</v>
@@ -6471,63 +6488,63 @@
         <v>2451</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>475</v>
+        <v>465</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>476</v>
+        <v>466</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>476</v>
+        <v>466</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>476</v>
+        <v>466</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>477</v>
+        <v>467</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>478</v>
+        <v>468</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>479</v>
+        <v>469</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>480</v>
+        <v>470</v>
       </c>
       <c r="R39" s="1" t="s">
-        <v>623</v>
+        <v>610</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>481</v>
+        <v>471</v>
       </c>
       <c r="T39" s="1" t="s">
-        <v>482</v>
+        <v>472</v>
       </c>
       <c r="U39" s="1" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
     </row>
-    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>483</v>
+        <v>473</v>
       </c>
       <c r="B40" s="7">
         <v>46083</v>
@@ -6536,63 +6553,63 @@
         <v>2452</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="P40" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="Q40" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="R40" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="S40" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="T40" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="I40" s="1" t="s">
+      <c r="U40" s="1" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
         <v>485</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="K40" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="L40" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="M40" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="N40" s="1" t="s">
-        <v>489</v>
-      </c>
-      <c r="O40" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="P40" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="Q40" s="1" t="s">
-        <v>624</v>
-      </c>
-      <c r="R40" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="S40" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="T40" s="1" t="s">
-        <v>494</v>
-      </c>
-      <c r="U40" s="1" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>495</v>
       </c>
       <c r="B41" s="7">
         <v>46083</v>
@@ -6601,63 +6618,63 @@
         <v>2504</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="O41" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="P41" s="1" t="s">
         <v>496</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="Q41" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>626</v>
-      </c>
-      <c r="G41" s="1" t="s">
+      <c r="R41" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="S41" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="T41" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="U41" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="K41" s="1" t="s">
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
         <v>502</v>
-      </c>
-      <c r="L41" s="1" t="s">
-        <v>503</v>
-      </c>
-      <c r="M41" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="N41" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="O41" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="P41" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="Q41" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="R41" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="S41" s="1" t="s">
-        <v>509</v>
-      </c>
-      <c r="T41" s="1" t="s">
-        <v>510</v>
-      </c>
-      <c r="U41" s="1" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>512</v>
       </c>
       <c r="B42" s="7">
         <v>46083</v>
@@ -6666,63 +6683,63 @@
         <v>2513</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>513</v>
+        <v>503</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>627</v>
+        <v>614</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>514</v>
+        <v>504</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>515</v>
+        <v>505</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>516</v>
+        <v>506</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>517</v>
+        <v>507</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>628</v>
+        <v>615</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>629</v>
+        <v>616</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>518</v>
+        <v>508</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="U42" s="1" t="s">
-        <v>630</v>
+        <v>617</v>
       </c>
     </row>
-    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="B43" s="7">
         <v>46083</v>
@@ -6731,63 +6748,63 @@
         <v>2545</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="S43" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="T43" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="U43" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
         <v>523</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="L43" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M43" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="N43" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O43" s="1" t="s">
-        <v>527</v>
-      </c>
-      <c r="P43" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="Q43" s="1" t="s">
-        <v>529</v>
-      </c>
-      <c r="R43" s="1" t="s">
-        <v>530</v>
-      </c>
-      <c r="S43" s="1" t="s">
-        <v>531</v>
-      </c>
-      <c r="T43" s="1" t="s">
-        <v>532</v>
-      </c>
-      <c r="U43" s="1" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>533</v>
       </c>
       <c r="B44" s="7">
         <v>46083</v>
@@ -6796,44 +6813,44 @@
         <v>3682</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
       <c r="O44" s="1" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>539</v>
+        <v>529</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="U44" s="1" t="s">
-        <v>631</v>
+        <v>618</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revising for symbols and formatting
</commit_message>
<xml_diff>
--- a/data/processed/pssi_form_data_altered.xlsx
+++ b/data/processed/pssi_form_data_altered.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\PSSI-final-tech-report\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A352C6-1346-4785-B4B8-3962E1484FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4831C3B-A3B3-4693-AC55-B6C40BC527ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -520,9 +520,6 @@
     <t>2407 PSSI Science Project Reporting Template_JessyBokvist_Final.docx</t>
   </si>
   <si>
-    <t>Characterizing juvenile Chinook salmon distribution, diet and health on the West Coast of Vancouver Island.</t>
-  </si>
-  <si>
     <t>Jessy Bokvist</t>
   </si>
   <si>
@@ -727,9 +724,6 @@
     <t>2413 PSSI Science Project Reporting BarkleyClayoquot.docx</t>
   </si>
   <si>
-    <t>Barkley Sound and Clayoquot Sound Krill Monitoring</t>
-  </si>
-  <si>
     <t>Akash Sastri, Kelly Young</t>
   </si>
   <si>
@@ -895,9 +889,6 @@
     <t>2418 PSSI Science Project Reporting-thiamine analysis-final-BC_EE.docx</t>
   </si>
   <si>
-    <t>Prediction of reproductive success of Chinook salmon based on Thiamine concentrations in returning adults</t>
-  </si>
-  <si>
     <t>Pacific Science Enterprise Centre</t>
   </si>
   <si>
@@ -919,9 +910,6 @@
   </si>
   <si>
     <t>2421 PSSI Science Project Reporting Johnson.docx</t>
-  </si>
-  <si>
-    <t>Measurement of stress hormones in scales and its application for the identification of conditions causing chronic stress in Pacific Salmon</t>
   </si>
   <si>
     <t>Stewart Johnson</t>
@@ -1522,9 +1510,6 @@
   </si>
   <si>
     <t>2439 PSSI Science Project Reporting.docx</t>
-  </si>
-  <si>
-    <t>Modernizing Fish Age Estimation using Fourier Transform-Near Infrared and Neural Network Techniques</t>
   </si>
   <si>
     <t>Stephen Wischniowski</t>
@@ -1675,9 +1660,6 @@
   </si>
   <si>
     <t>2447 PSSI Reporting - Fit-Chips and eDNA Project .docx</t>
-  </si>
-  <si>
-    <t>Innovative Ecosystem Based Approaches to identify cumulative stressors: Salmon Fit-Chips and eDNA</t>
   </si>
   <si>
     <t>Kristi Saunders (retired), Christoph Deeg, Arthur Bass, Carl Llewellyn</t>
@@ -1774,9 +1756,6 @@
     <t>2448 PSSI_Science_Project_Reporting.docx</t>
   </si>
   <si>
-    <t>Developing a proactive, modernized, holistic approach to ensure optimal health and condition of Hatchery Production.</t>
-  </si>
-  <si>
     <t>Christoph Deeg, Kristi Miller-Saunders (retired), Karia Kaukinen, Arthur Bass</t>
   </si>
   <si>
@@ -2272,10 +2251,6 @@
 Figure 2. Maps of Clayoquot Sound showing the percentage of the top 5m of the water column exceeding 17Â°C in summer (July, August and September) in the (a) simulation for 2024 and (b) future scenario. Panel (c) shows the difference between both (future scenario minus 2024 simulation), highlighting the additional percentage of the surface waters that can exceed the temperature threshold in the future scenario.
 Figure 3. Time series of the percentage of water volume that exceeds 17Â°C in Tofino inlet at different depth ranges and different simulations. Bold colours indicate the future scenario, while paler colours indicate the 2024 simulation. Green colours indicate the volume in the surface depth range (0 to 5 m), blue colours represent upper waters below the surface (5 to 20 m) and black/grey represent deep waters (20 to 100 m). At surface, both simulations exceed the threshold between spring and autumn, while below 5 m the threshold is exceeded mostly in the future scenario.
 Figure 4. Location of the CTD profiles with oxygen data from 2024. The oxygen histograms show the distribution of oxygen data for the whole 2024 year and four seasons (winter: Jan-Mar, spring: Apr-Jun, summer: Jul-Sep, and winter: Oct-Dec). The different colours show the histograms for four different depth ranges: the whole water column (blue), top 50 meters (orange), top 20 meters (yellow) and top 5 meters (purple).</t>
-  </si>
-  <si>
-    <t>Rosen, S., Bianucci, L., Jackson, J.M., Hare, A., Greengrove, C., Monks, R., Bartlett, M. and Dick, J., 2022. Seasonal near-surface hypoxia in a temperate fjord in Clayoquot Sound, British Columbia.Â *Frontiers in Marine Science*,Â *9*, p.1000041.
-Foreman, M.G.G., Chandler, P.C., Bianucci, L., Wan, D., Krassovski, M.V., Thupaki, P., Cooper, G. and Lin, Y., 2024. A circulation model for inlets along the central West Coast of Vancouver Island.Â *Atmosphere-Ocean*,Â *62*(1), pp.58-89.</t>
   </si>
   <si>
     <t>*Overview of the model*
@@ -2550,32 +2525,6 @@
     <t>Province of British Columbia, Pacific Salmon Commission</t>
   </si>
   <si>
-    <t>Chan, F.T., Beatty, S.J., Gilles Jr, A.S., Hill, J.E., Kozic, S., Luo, D., Morgan, D.L., Pavia Jr, R.T., Therriault, T.W., Verreycken, H. and Vilizzi, L., 2019. Leaving the fish bowl: the ornamental trade as a global vector for freshwater fish invasions.Â *Aquatic Ecosystem Health &amp; Management*,Â *22*(4), pp.417-439.
-Deacon, J.E., Hubbs, C. and Zahuranec, B.J., 1964. Some effects of introduced fishes on the native fish fauna of southern Nevada.Â *Copeia*, pp.384-388.
-Dextrase, A.J. and Mandrak, N.E., 2006. Impacts of alien invasive species on freshwater fauna at risk in Canada.Â *Biological Invasions*,Â *8*(1), pp.13-24.
-Egertson, C.J. and Downing, J.A., 2004. Relationship of fish catch and composition to water quality in a suite of agriculturally eutrophic lakes.Â *Canadian Journal of Fisheries and Aquatic Sciences*,Â *61*(9), pp.1784-1796.
-Faisal, M., Shavalier, M., Kim, R.K., Millard, E.V., Gunn, M.R., Winters, A.D., Schulz, C.A., Eissa, A., Thomas, M.V., Wolgamood, M. and Whelan, G.E., 2012. Spread of the emerging viral hemorrhagic septicemia virus strain, genotype IVb, in Michigan, USA.Â *Viruses*,Â *4*(5), pp.734-760.
-Gilad, O., Yun, S., Zagmutt-Vergara, F.J., Leutenegger, C.M., Bercovier, H. and Hedrick, R.P., 2004. Concentrations of a Koi herpesvirus (KHV) in tissues of experimentally-infected Cyprinus carpio koi as assessed by real-time TaqMan PCR.Â *Diseases of aquatic organisms*,Â *60*, pp.179-187.
-Jackson, Z.J., Quist, M.C., Downing, J.A. and Larscheid, J.G., 2010. Common carp (Cyprinus carpio), sport fishes, and water quality: ecological thresholds in agriculturally eutrophic lakes.Â *Lake and Reservoir Management*,Â *26*(1), pp.14-22.
-Jalbert, C.S., Falke, J.A., LÃ³pez, J.A., Dunker, K.J., Sepulveda, A.J. and Westley, P.A., 2021. Vulnerability of Pacific salmon to invasion of northern pike (Esox lucius) in Southcentral Alaska.Â *PLoS One*,Â *16*(7), p.e0254097.
-Jones, P.W. and Martin, F.D., 1978.Â *Development of Fishes of the Mid-Atlantic Bight: Acipenseridae Through Ictaluridae*. pp 323.
-Lentsch, L.D., Muth, R., Thompson, P.D., Crowl, T.A. and Hoskins, B.G., 1996. Options for selectively controlling non-indigenous fish in the Upper Colorado River Basin.Â *Final Report. Publication*, pp.96-14.
-Marsh, P.C. and Douglas, M.E., 1997. Predation by introduced fishes on endangered humpback chub and other native species in the Little Colorado River, Arizona.Â *Transactions of the American Fisheries Society*,Â *126*(2), pp.343-346.
-Miller, A.I. and Beckman, L.G., 1996. First record of predation on white sturgeon eggs by sympatric fishes.Â *Transactions of the American Fisheries Society*,Â *125*(2), pp.338-340.
-Moyle, P.B. 1976. Inland fishes of California. University of California Press, Berkeley, CA.
-Nowosad, D.M. and Taylor, E.B., 2013. Habitat variation and invasive species as factors influencing the distribution of native fishes in the lower Fraser River Valley, British Columbia, with an emphasis on brassy minnow (*Hybognathus hankinsoni*).Â *Canadian journal of zoology*,Â *91*(2), pp.71-81.
-Poelen, J.H., Simons, J.D. and Mungall, C.J., 2014. Global biotic interactions: An open infrastructure to share and analyze species-interaction datasets.Â *Ecological informatics*,Â *24*, pp.148-159.
-Richardson, M.J., Whoriskey, F.G. and Roy, L.H., 1995. Turbidity generation and biological impacts of an exotic fish Carassius auratus, introduced into shallow seasonally anoxic ponds.Â *Journal of fish biology*,Â *47*(4), pp.576-585.
-Robinette, H.R. and Knight, S.S., 1981. Food of channel catfish during flooding of the Tombigbee River, Mississippi. InÂ *Proceedings of the Southeastern Association of Fish and Wildlife Agencies*Â (Vol. 35, pp. 598-606).
-Sala, O.E., Stuart Chapin, F.I.I.I., Armesto, J.J., Berlow, E., Bloomfield, J., Dirzo, R., Huber-Sanwald, E., Huenneke, L.F., Jackson, R.B., Kinzig, A. and Leemans, R., 2000. Global biodiversity scenarios for the year 2100.Â *science*,Â *287*(5459), pp.1770-1774.
-Sanderson, B.L., Barnas, K.A. and Rub, A.M.W., 2009. Nonindigenous species of the Pacific Northwest: an overlooked risk to endangered salmon?.Â *BioScience*,Â *59*(3), pp.245-256.
-Schwoerer, T., Little, J.M. and Adkison, M.D., 2019. Aquatic invasive species change ecosystem services from the world's largest wild sockeye salmon fisheries in Alaska.Â *Journal of Ocean and Coastal Economics*,Â *6*(1), p.2.
-Scott, W.B., 1973. Freshwater fishes of Canada.Â *Fish. Res. Board Can. Bull.*,Â *184*, pp.1-966.
-Vigg, S., Poe, T.P., Prendergast, L.A. and Hansel, H.C., 1991. Rates of consumption of juvenile salmonids and alternative prey fish by northern squawfish, walleyes, smallmouth bass, and channel catfish in John Day Reservoir, Columbia River.Â *Transactions of the American Fisheries Society*,Â *120*(4), pp.421-438.
-Weber, M.J. and Brown, M.L., 2009. Effects of common carp on aquatic ecosystems 80 years after "carp as a dominant": ecological insights for fisheries management.Â *Reviews in Fisheries Science*,Â *17*(4), pp.524-537.
-Wilcox, M.A., Johnson, D., Dyke, K., Gunsch, D., Lyons, D.A., DiBacco, C. and Therriault, T.W., 2025. Identifying higher risk invaders to the Columbia Glaciated Freshwater Ecoregion using a new screening tool: the Non-Indigenous Species Screening Tool (NISST).Â *Management of Biological Invasions*,Â *16*(1), pp.187-210.</t>
-  </si>
-  <si>
     <t>Under global climate change, co-occurrence of gradual physical changes in seawater and extreme events pose a substantial threat to marine ecosystems (IPCC, 2023). This PSSI-funded project focused on the Strait of Georgia (SOG) within the Northeast Pacific coastal region where steady rises in mean seasonal seawater temperatures and *p*CO2 levels, and increasingly prevalent acute stressor events such as heatwaves and low-pH upwellings, are already occurring (Bylhouwer et al., 2013; Evans et al., 2019; Okey et al., 2024; Raymond et al., 2022; Talloni-Alvarez et al., 2014). Moreover, the SOG is distinctive as conditions of high *p*CO2 and aragonite undersaturation persist year-round across a wide extent of the water column (Moore-Maley et al., 2016; Simpson et al., 2024). *Limacina helicina*, a cold-water pteropod well-represented within the region's zooplankton communities, is highly susceptible to climate change stressors, with documented impacts of ocean warming and ocean acidification (OA) on shell development, growth, and survival (BednarÅ¡ek et al., 2016, 2022; Lischka et al., 2022; Lischka &amp; Riebesell, 2012). However, there has been minimal investigation of climate change effects on the species' nutritional status (*e.g.* fatty acid (FA) composition) under regionally-relevant conditions. Given the importance of *L. helicina* as a dietary item for some populations of juvenile Pacific salmon species in the Northeast Pacific (Brodeur et al., 2007; Doubleday &amp; Hopcroft, 2015; Sturdevant et al., 2012), it was proposed that any change in the nutritive status of *L. helicina* under climate stressor conditions could have carry-over impacts to juvenile salmon growth, health, and survival.
 The project involved cross-program collaboration between DFO researchers based at the Pacific Biological Station (PBS) and the Pacific Science Enterprise Centre (PSEC) for investigation of the impacts of warming and OA conditions (representative of future conditions in the SOG) on FA profiles of *L. helicina* populations in the region. *Limacina helicina* samples were collected and processed as part of juvenile Pacific salmon survey fieldwork carried out in the SOG during 2014âˆ’2023 by the *Salmon Marine Interactions Program* at PBS (Lead: Neville). The program also supported live collection (within the SOG) of *L. helicina* for a climate change experiment (2023). Subsequent field sample sorting (*i.e.* extraction of whole pteropods from historical size-fractionated plankton samples) and laboratory experimentation (*i.e.* conducting of a climate change experiment in the Fisheries and Oceans Climate Change and Ocean Acidification Laboratory (FOCCOAL)), and nutritional analyses (*i.e.* FA analyses via gas chromatography) were carried out by the *Sustainable Invertebrate Aquaculture Program* at PBS (Lead: Pearce) and *Nutrition Program* at PSEC (Lead: Forster), respectively.</t>
   </si>
@@ -3197,9 +3146,6 @@
     <t>Enhanced Mark Selective Fishery (MSF) monitoring (including a Chinook Reference Fishery)</t>
   </si>
   <si>
-    <t>Assessment of SEP Chinook and coho broodstock ELISA screening data by modelling for explanatory variables, and yearling DFAT prevalence data by modelling for predictive variables.</t>
-  </si>
-  <si>
     <t>Epidemiological modeling of infectious hematopoietic necrosis virus in sockeye salmon</t>
   </si>
   <si>
@@ -3207,6 +3153,60 @@
   </si>
   <si>
     <t>Improvement, expansion and modernization of salmonid health diagnostic services for optimizing salmonid hatchery health management</t>
+  </si>
+  <si>
+    <t>Barkley Sound and Clayoquot Sound krill monitoring</t>
+  </si>
+  <si>
+    <t>Prediction of reproductive success of Chinook salmon based on thiamine concentrations in returning adults</t>
+  </si>
+  <si>
+    <t>Measurement of stress hormones in scales and its application for the identification of conditions causing chronic stress in Pacific salmon</t>
+  </si>
+  <si>
+    <t>Modernizing fish age estimation using Fourier transform-near infrared and neural network techniques</t>
+  </si>
+  <si>
+    <t>Innovative ecosystem based approaches to identify cumulative stressors: Salmon Fit-Chips and eDNA</t>
+  </si>
+  <si>
+    <t>Developing a proactive, modernized, holistic approach to ensure optimal health and condition of hatchery production</t>
+  </si>
+  <si>
+    <t>Assessment of SEP Chinook and coho broodstock ELISA screening data by modelling for explanatory variables, and yearling DFAT prevalence data by modelling for predictive variables</t>
+  </si>
+  <si>
+    <t>Characterizing juvenile Chinook salmon distribution, diet and health on the West Coast of Vancouver Island</t>
+  </si>
+  <si>
+    <t>Chan, F.T., Beatty, S.J., Gilles Jr, A.S., Hill, J.E., Kozic, S., Luo, D., Morgan, D.L., Pavia Jr, R.T., Therriault, T.W., Verreycken, H. and Vilizzi, L., 2019. Leaving the fish bowl: the ornamental trade as a global vector for freshwater fish invasions. Aquatic Ecosystem Health &amp; Management, 22(4), pp.417-439.
+Deacon, J.E., Hubbs, C. and Zahuranec, B.J., 1964. Some effects of introduced fishes on the native fish fauna of southern Nevada. Copeia, pp.384-388.
+Dextrase, A.J. and Mandrak, N.E., 2006. Impacts of alien invasive species on freshwater fauna at risk in Canada. Biological Invasions, 8(1), pp.13-24.
+Egertson, C.J. and Downing, J.A., 2004. Relationship of fish catch and composition to water quality in a suite of agriculturally eutrophic lakes. Canadian Journal of Fisheries and Aquatic Sciences, 61(9), pp.1784-1796.
+Faisal, M., Shavalier, M., Kim, R.K., Millard, E.V., Gunn, M.R., Winters, A.D., Schulz, C.A., Eissa, A., Thomas, M.V., Wolgamood, M. and Whelan, G.E., 2012. Spread of the emerging viral hemorrhagic septicemia virus strain, genotype IVb, in Michigan, USA. Viruses, 4(5), pp.734-760.
+Gilad, O., Yun, S., Zagmutt-Vergara, F.J., Leutenegger, C.M., Bercovier, H. and Hedrick, R.P., 2004. Concentrations of a Koi herpesvirus (KHV) in tissues of experimentally-infected Cyprinus carpio koi as assessed by real-time TaqMan PCR. Diseases of aquatic organisms, 60, pp.179-187.
+Jackson, Z.J., Quist, M.C., Downing, J.A. and Larscheid, J.G., 2010. Common carp (Cyprinus carpio), sport fishes, and water quality: ecological thresholds in agriculturally eutrophic lakes. Lake and Reservoir Management, 26(1), pp.14-22.
+Jalbert, C.S., Falke, J.A., López, J.A., Dunker, K.J., Sepulveda, A.J. and Westley, P.A., 2021. Vulnerability of Pacific salmon to invasion of northern pike (Esox lucius) in Southcentral Alaska. PLoS One, 16(7), p.e0254097.
+Jones, P.W. and Martin, F.D., 1978. Development of Fishes of the Mid-Atlantic Bight: Acipenseridae Through Ictaluridae. pp 323. 
+Lentsch, L.D., Muth, R., Thompson, P.D., Crowl, T.A. and Hoskins, B.G., 1996. Options for selectively controlling non-indigenous fish in the Upper Colorado River Basin. Final Report. Publication, pp.96-14.
+Marsh, P.C. and Douglas, M.E., 1997. Predation by introduced fishes on endangered humpback chub and other native species in the Little Colorado River, Arizona. Transactions of the American Fisheries Society, 126(2), pp.343-346.
+Miller, A.I. and Beckman, L.G., 1996. First record of predation on white sturgeon eggs by sympatric fishes. Transactions of the American Fisheries Society, 125(2), pp.338-340.
+Moyle, P.B. 1976. Inland fishes of California. University of California Press, Berkeley, CA.
+Nowosad, D.M. and Taylor, E.B., 2013. Habitat variation and invasive species as factors influencing the distribution of native fishes in the lower Fraser River Valley, British Columbia, with an emphasis on brassy minnow (Hybognathus hankinsoni). Canadian journal of zoology, 91(2), pp.71-81.
+Poelen, J.H., Simons, J.D. and Mungall, C.J., 2014. Global biotic interactions: An open infrastructure to share and analyze species-interaction datasets. Ecological informatics, 24, pp.148-159.
+Richardson, M.J., Whoriskey, F.G. and Roy, L.H., 1995. Turbidity generation and biological impacts of an exotic fish Carassius auratus, introduced into shallow seasonally anoxic ponds. Journal of fish biology, 47(4), pp.576-585.
+Robinette, H.R. and Knight, S.S., 1981. Food of channel catfish during flooding of the Tombigbee River, Mississippi. In Proceedings of the Southeastern Association of Fish and Wildlife Agencies (Vol. 35, pp. 598-606).
+Sala, O.E., Stuart Chapin, F.I.I.I., Armesto, J.J., Berlow, E., Bloomfield, J., Dirzo, R., Huber-Sanwald, E., Huenneke, L.F., Jackson, R.B., Kinzig, A. and Leemans, R., 2000. Global biodiversity scenarios for the year 2100. science, 287(5459), pp.1770-1774.
+Sanderson, B.L., Barnas, K.A. and Rub, A.M.W., 2009. Nonindigenous species of the Pacific Northwest: an overlooked risk to endangered salmon?. BioScience, 59(3), pp.245-256.
+Schwoerer, T., Little, J.M. and Adkison, M.D., 2019. Aquatic invasive species change ecosystem services from the world's largest wild sockeye salmon fisheries in Alaska. Journal of Ocean and Coastal Economics, 6(1), p.2.
+Scott, W.B., 1973. Freshwater fishes of Canada. Fish. Res. Board Can. Bull., 184, pp.1-966.
+Vigg, S., Poe, T.P., Prendergast, L.A. and Hansel, H.C., 1991. Rates of consumption of juvenile salmonids and alternative prey fish by northern squawfish, walleyes, smallmouth bass, and channel catfish in John Day Reservoir, Columbia River. Transactions of the American Fisheries Society, 120(4), pp.421-438.
+Weber, M.J. and Brown, M.L., 2009. Effects of common carp on aquatic ecosystems 80 years after “carp as a dominant”: ecological insights for fisheries management. Reviews in Fisheries Science, 17(4), pp.524-537.
+Wilcox, M.A., Johnson, D., Dyke, K., Gunsch, D., Lyons, D.A., DiBacco, C. and Therriault, T.W., 2025. Identifying higher risk invaders to the Columbia Glaciated Freshwater Ecoregion using a new screening tool: the Non-Indigenous Species Screening Tool (NISST). Management of Biological Invasions, 16(1), pp.187-210.</t>
+  </si>
+  <si>
+    <t>Rosen, S., Bianucci, L., Jackson, J.M., Hare, A., Greengrove, C., Monks, R., Bartlett, M. and Dick, J., 2022. Seasonal near-surface hypoxia in a temperate fjord in Clayoquot Sound, British Columbia. Frontiers in Marine Science, 9, p.1000041.
+Foreman, M.G.G., Chandler, P.C., Bianucci, L., Wan, D., Krassovski, M.V., Thupaki, P., Cooper, G. and Lin, Y., 2024. A circulation model for inlets along the central West Coast of Vancouver Island. Atmosphere-Ocean, 62(1), pp.58-89.</t>
   </si>
 </sst>
 </file>
@@ -3263,7 +3263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3274,6 +3274,9 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4021,7 +4024,7 @@
     <col min="18" max="18" width="11.42578125" style="2"/>
     <col min="19" max="19" width="12.85546875" style="2" customWidth="1"/>
     <col min="20" max="20" width="15.7109375" style="2" customWidth="1"/>
-    <col min="21" max="21" width="12.7109375" style="2" customWidth="1"/>
+    <col min="21" max="21" width="126.85546875" style="10" customWidth="1"/>
     <col min="22" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
@@ -4086,7 +4089,7 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="10" t="s">
         <v>20</v>
       </c>
     </row>
@@ -4101,7 +4104,7 @@
         <v>22</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>636</v>
+        <v>627</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -4131,7 +4134,7 @@
         <v>31</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>32</v>
@@ -4181,7 +4184,7 @@
         <v>44</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>45</v>
@@ -4190,13 +4193,13 @@
         <v>46</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>47</v>
@@ -4237,7 +4240,7 @@
         <v>55</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>56</v>
@@ -4246,7 +4249,7 @@
         <v>57</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>58</v>
@@ -4258,19 +4261,19 @@
         <v>59</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>536</v>
+        <v>529</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>60</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="R4" s="1" t="s">
         <v>61</v>
@@ -4279,10 +4282,10 @@
         <v>62</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>538</v>
+        <v>531</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -4296,16 +4299,16 @@
         <v>2401</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>638</v>
+        <v>628</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>64</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>65</v>
@@ -4337,7 +4340,7 @@
         <v>72</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
@@ -4378,7 +4381,7 @@
         <v>81</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>82</v>
@@ -4390,7 +4393,7 @@
         <v>84</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>85</v>
@@ -4416,7 +4419,7 @@
         <v>2403</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>639</v>
+        <v>629</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>90</v>
@@ -4437,7 +4440,7 @@
         <v>95</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="L7" s="4" t="s">
         <v>96</v>
@@ -4446,7 +4449,7 @@
         <v>96</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>97</v>
@@ -4455,84 +4458,84 @@
         <v>98</v>
       </c>
       <c r="Q7" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>616</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" s="8">
+        <v>46083</v>
+      </c>
+      <c r="C8" s="4">
+        <v>2404</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="R7" s="4" t="s">
-        <v>534</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>625</v>
-      </c>
-      <c r="T7" s="4" t="s">
-        <v>534</v>
-      </c>
-      <c r="U7" s="4" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B8" s="7">
-        <v>46083</v>
-      </c>
-      <c r="C8" s="1">
-        <v>2404</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="I8" s="1" t="s">
+      <c r="H8" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="K8" s="1" t="s">
+      <c r="J8" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="L8" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O8" s="1" t="s">
+      <c r="L8" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="O8" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="1" t="s">
+      <c r="P8" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="Q8" s="1" t="s">
-        <v>542</v>
-      </c>
-      <c r="R8" s="1" t="s">
+      <c r="Q8" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="R8" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="S8" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="T8" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>544</v>
+      <c r="T8" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="U8" s="5" t="s">
+        <v>640</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
@@ -4549,19 +4552,19 @@
         <v>110</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>111</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>112</v>
@@ -4570,13 +4573,13 @@
         <v>113</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>114</v>
@@ -4585,7 +4588,7 @@
         <v>115</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="R9" s="1" t="s">
         <v>116</v>
@@ -4597,7 +4600,7 @@
         <v>118</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
@@ -4617,40 +4620,40 @@
         <v>121</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>122</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>124</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>533</v>
+        <v>526</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>125</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="R10" s="1" t="s">
         <v>126</v>
@@ -4675,64 +4678,64 @@
       <c r="C11" s="4">
         <v>2407</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>634</v>
-      </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="I11" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="J11" s="4" t="s">
         <v>135</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>136</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>56</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N11" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="O11" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="O11" s="4" t="s">
+      <c r="P11" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="P11" s="4" t="s">
+      <c r="Q11" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="Q11" s="4" t="s">
+      <c r="R11" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="R11" s="4" t="s">
+      <c r="S11" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="S11" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="T11" s="4" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="7">
         <v>46083</v>
@@ -4741,19 +4744,19 @@
         <v>2408</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>640</v>
+        <v>630</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>550</v>
+        <v>542</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>56</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
@@ -4763,35 +4766,35 @@
         <v>56</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="P12" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="P12" s="1" t="s">
+      <c r="Q12" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="R12" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="Q12" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="R12" s="1" t="s">
+      <c r="S12" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="S12" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="T12" s="1" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>553</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B13" s="7">
         <v>46083</v>
@@ -4800,61 +4803,61 @@
         <v>2409</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I13" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="M13" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N13" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="M13" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N13" s="1" t="s">
+      <c r="O13" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="O13" s="1" t="s">
+      <c r="P13" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="P13" s="1" t="s">
+      <c r="Q13" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="Q13" s="1" t="s">
+      <c r="R13" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="R13" s="1" t="s">
+      <c r="S13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="S13" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="T13" s="1" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B14" s="7">
         <v>46083</v>
@@ -4863,22 +4866,22 @@
         <v>2410</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="F14" s="1" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>31</v>
@@ -4890,36 +4893,36 @@
         <v>31</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="O14" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="P14" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="P14" s="1" t="s">
+      <c r="Q14" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="Q14" s="1" t="s">
+      <c r="R14" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="R14" s="1" t="s">
+      <c r="S14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="S14" s="1" t="s">
+      <c r="T14" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="T14" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>557</v>
+      <c r="U14" s="5" t="s">
+        <v>639</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B15" s="7">
         <v>46083</v>
@@ -4928,63 +4931,63 @@
         <v>2412</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>629</v>
+        <v>620</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>178</v>
-      </c>
       <c r="J15" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>56</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O15" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="R15" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="P15" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>559</v>
-      </c>
-      <c r="R15" s="1" t="s">
+      <c r="S15" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="S15" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="T15" s="1" t="s">
-        <v>560</v>
+        <v>551</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>561</v>
+        <v>552</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B16" s="7">
         <v>46083</v>
@@ -4992,64 +4995,64 @@
       <c r="C16" s="1">
         <v>2413</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="9" t="s">
+        <v>631</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="F16" s="1" t="s">
-        <v>562</v>
-      </c>
-      <c r="G16" s="1" t="s">
+      <c r="I16" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="J16" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="I16" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="J16" s="1" t="s">
+      <c r="L16" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O16" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="P16" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="L16" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N16" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O16" s="1" t="s">
+      <c r="Q16" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="P16" s="1" t="s">
+      <c r="R16" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="Q16" s="1" t="s">
+      <c r="S16" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="R16" s="1" t="s">
+      <c r="T16" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="U16" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="S16" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>563</v>
-      </c>
-      <c r="U16" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B17" s="7">
         <v>46083</v>
@@ -5058,63 +5061,63 @@
         <v>2416</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="G17" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>564</v>
-      </c>
-      <c r="G17" s="1" t="s">
+      <c r="I17" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>104</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="M17" s="1" t="s">
         <v>104</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>565</v>
+        <v>556</v>
       </c>
       <c r="P17" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="R17" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="Q17" s="1" t="s">
+      <c r="S17" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="R17" s="1" t="s">
+      <c r="T17" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="S17" s="1" t="s">
+      <c r="U17" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="T17" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B18" s="7">
         <v>46083</v>
@@ -5123,63 +5126,63 @@
         <v>2417</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="I18" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="J18" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="I18" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="J18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="M18" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O18" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="P18" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="M18" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O18" s="1" t="s">
+      <c r="Q18" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="S18" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="P18" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="Q18" s="1" t="s">
-        <v>566</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>567</v>
-      </c>
-      <c r="S18" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="T18" s="1" t="s">
-        <v>568</v>
+        <v>559</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>569</v>
+        <v>560</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B19" s="7">
         <v>46083</v>
@@ -5187,64 +5190,64 @@
       <c r="C19" s="1">
         <v>2418</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="J19" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="G19" s="1" t="s">
+      <c r="K19" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="L19" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="M19" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O19" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="I19" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="J19" s="1" t="s">
+      <c r="P19" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="S19" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O19" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>571</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="S19" s="1" t="s">
-        <v>228</v>
-      </c>
       <c r="T19" s="5" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>574</v>
+        <v>565</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B20" s="7">
         <v>46083</v>
@@ -5252,64 +5255,64 @@
       <c r="C20" s="1">
         <v>2421</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>230</v>
+      <c r="D20" s="9" t="s">
+        <v>633</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>575</v>
+        <v>566</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>56</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>577</v>
+        <v>568</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B21" s="7">
         <v>46083</v>
@@ -5318,63 +5321,63 @@
         <v>2422</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>579</v>
+        <v>570</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>104</v>
       </c>
       <c r="L21" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="R21" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="M21" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O21" s="1" t="s">
+      <c r="S21" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="P21" s="1" t="s">
+      <c r="T21" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="Q21" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="R21" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="S21" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>248</v>
-      </c>
       <c r="U21" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B22" s="7">
         <v>46083</v>
@@ -5383,63 +5386,63 @@
         <v>2424</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>626</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="J22" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="K22" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="F22" s="9" t="s">
-        <v>635</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="H22" s="1" t="s">
+      <c r="L22" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O22" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="P22" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="R22" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="S22" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="T22" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="L22" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>582</v>
-      </c>
-      <c r="R22" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="S22" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="U22" s="1" t="s">
-        <v>583</v>
+        <v>574</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B23" s="7">
         <v>46083</v>
@@ -5448,63 +5451,63 @@
         <v>2425</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>623</v>
+        <v>614</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="K23" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="F23" s="9" t="s">
-        <v>534</v>
-      </c>
-      <c r="G23" s="1" t="s">
+      <c r="L23" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N23" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="O23" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="I23" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="J23" s="1" t="s">
+      <c r="P23" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="Q23" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="L23" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N23" s="1" t="s">
+      <c r="R23" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="O23" s="1" t="s">
+      <c r="S23" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="P23" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="R23" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="S23" s="1" t="s">
-        <v>271</v>
-      </c>
       <c r="T23" s="1" t="s">
-        <v>584</v>
+        <v>575</v>
       </c>
       <c r="U23" s="1" t="s">
-        <v>585</v>
+        <v>576</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B24" s="7">
         <v>46083</v>
@@ -5513,63 +5516,63 @@
         <v>2426</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>618</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="F24" s="9" t="s">
-        <v>627</v>
-      </c>
-      <c r="G24" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="L24" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="M24" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="N24" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="O24" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="L24" s="1" t="s">
+      <c r="P24" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="R24" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="M24" s="1" t="s">
+      <c r="S24" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="N24" s="1" t="s">
+      <c r="T24" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="O24" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="P24" s="1" t="s">
-        <v>586</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="R24" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="S24" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="U24" s="1" t="s">
-        <v>588</v>
+        <v>579</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B25" s="7">
         <v>46083</v>
@@ -5578,63 +5581,63 @@
         <v>2427</v>
       </c>
       <c r="D25" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O25" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="G25" s="1" t="s">
+      <c r="P25" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="J25" s="1" t="s">
+      <c r="Q25" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="R25" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="S25" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="L25" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O25" s="1" t="s">
+      <c r="T25" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="P25" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="Q25" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="R25" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="S25" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>295</v>
-      </c>
       <c r="U25" s="1" t="s">
-        <v>590</v>
+        <v>581</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B26" s="7">
         <v>46083</v>
@@ -5643,63 +5646,63 @@
         <v>2430</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>619</v>
+        <v>610</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="L26" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>591</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="M26" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="P26" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="S26" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="L26" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>620</v>
-      </c>
-      <c r="Q26" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="R26" s="1" t="s">
-        <v>621</v>
-      </c>
-      <c r="S26" s="1" t="s">
-        <v>304</v>
-      </c>
       <c r="T26" s="1" t="s">
-        <v>622</v>
+        <v>613</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B27" s="7">
         <v>46083</v>
@@ -5708,63 +5711,63 @@
         <v>2432</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>624</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="P27" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="Q27" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="E27" s="9" t="s">
-        <v>633</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>593</v>
-      </c>
-      <c r="G27" s="1" t="s">
+      <c r="R27" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M27" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N27" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O27" s="1" t="s">
+      <c r="S27" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="P27" s="1" t="s">
+      <c r="T27" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="Q27" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="R27" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="S27" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="T27" s="1" t="s">
-        <v>313</v>
-      </c>
       <c r="U27" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B28" s="7">
         <v>46083</v>
@@ -5773,63 +5776,63 @@
         <v>2433</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>624</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="P28" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q28" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="E28" s="9" t="s">
-        <v>633</v>
-      </c>
-      <c r="F28" s="1" t="s">
+      <c r="R28" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="S28" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="K28" s="9" t="s">
-        <v>534</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N28" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O28" s="1" t="s">
-        <v>594</v>
-      </c>
-      <c r="P28" s="1" t="s">
+      <c r="T28" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="Q28" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="R28" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="S28" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="T28" s="1" t="s">
-        <v>322</v>
-      </c>
       <c r="U28" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B29" s="7">
         <v>46083</v>
@@ -5838,63 +5841,63 @@
         <v>2434</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I29" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="J29" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="K29" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="L29" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="M29" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="I29" s="1" t="s">
+      <c r="N29" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="O29" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="P29" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="L29" s="1" t="s">
+      <c r="Q29" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="M29" s="1" t="s">
+      <c r="R29" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="N29" s="1" t="s">
+      <c r="S29" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="O29" s="1" t="s">
-        <v>595</v>
-      </c>
-      <c r="P29" s="1" t="s">
+      <c r="T29" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="Q29" s="1" t="s">
+      <c r="U29" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="R29" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="S29" s="1" t="s">
-        <v>336</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="U29" s="1" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="B30" s="7">
         <v>46083</v>
@@ -5903,63 +5906,63 @@
         <v>2435</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>630</v>
+        <v>621</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="K30" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="L30" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="M30" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="N30" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="O30" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="P30" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="M30" s="1" t="s">
+      <c r="Q30" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="N30" s="1" t="s">
+      <c r="R30" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="O30" s="1" t="s">
+      <c r="S30" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="P30" s="1" t="s">
+      <c r="T30" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="Q30" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="R30" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>355</v>
-      </c>
       <c r="U30" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B31" s="7">
         <v>46083</v>
@@ -5968,63 +5971,63 @@
         <v>2436</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="G31" s="1" t="s">
+      <c r="K31" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="L31" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N31" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="O31" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="P31" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="K31" s="1" t="s">
+      <c r="Q31" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="L31" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N31" s="1" t="s">
+      <c r="R31" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="O31" s="1" t="s">
+      <c r="S31" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="P31" s="1" t="s">
+      <c r="T31" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="Q31" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="T31" s="1" t="s">
-        <v>370</v>
-      </c>
       <c r="U31" s="1" t="s">
-        <v>596</v>
+        <v>587</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B32" s="7">
         <v>46083</v>
@@ -6033,63 +6036,63 @@
         <v>2437</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="J32" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="F32" s="1" t="s">
-        <v>597</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="H32" s="1" t="s">
+      <c r="L32" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="I32" s="1" t="s">
+      <c r="M32" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="N32" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="O32" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="P32" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="L32" s="1" t="s">
+      <c r="Q32" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="M32" s="1" t="s">
+      <c r="R32" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="N32" s="1" t="s">
+      <c r="S32" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="O32" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="P32" s="1" t="s">
+      <c r="T32" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="Q32" s="1" t="s">
+      <c r="U32" s="1" t="s">
         <v>382</v>
-      </c>
-      <c r="R32" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="B33" s="7">
         <v>46083</v>
@@ -6097,64 +6100,64 @@
       <c r="C33" s="1">
         <v>2439</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="P33" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="Q33" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>599</v>
-      </c>
-      <c r="G33" s="1" t="s">
+      <c r="R33" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="S33" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="K33" s="1" t="s">
+      <c r="T33" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="L33" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="P33" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="Q33" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="R33" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>397</v>
-      </c>
       <c r="U33" s="1" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="B34" s="7">
         <v>46083</v>
@@ -6163,63 +6166,63 @@
         <v>2442</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="L34" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="M34" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="N34" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>602</v>
-      </c>
-      <c r="G34" s="1" t="s">
+      <c r="O34" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="H34" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="J34" s="1" t="s">
+      <c r="P34" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="K34" s="1" t="s">
+      <c r="Q34" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="R34" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="L34" s="1" t="s">
+      <c r="S34" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="M34" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="N34" s="1" t="s">
+      <c r="T34" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="O34" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="P34" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>603</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>410</v>
-      </c>
       <c r="U34" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="B35" s="7">
         <v>46083</v>
@@ -6227,64 +6230,64 @@
       <c r="C35" s="1">
         <v>2443</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>412</v>
+      <c r="D35" s="9" t="s">
+        <v>407</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>604</v>
+        <v>595</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I35" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="P35" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="Q35" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="R35" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="K35" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="N35" s="1" t="s">
+      <c r="S35" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="O35" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>422</v>
-      </c>
       <c r="T35" s="1" t="s">
-        <v>605</v>
+        <v>596</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="B36" s="7">
         <v>46083</v>
@@ -6292,26 +6295,26 @@
       <c r="C36" s="1">
         <v>2447</v>
       </c>
-      <c r="D36" s="1" t="s">
-        <v>424</v>
+      <c r="D36" s="9" t="s">
+        <v>635</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>606</v>
+        <v>597</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>78</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>104</v>
@@ -6320,36 +6323,36 @@
         <v>104</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N36" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="S36" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="T36" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="O36" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="P36" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="Q36" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="R36" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="S36" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="T36" s="1" t="s">
-        <v>434</v>
-      </c>
       <c r="U36" s="1" t="s">
-        <v>607</v>
+        <v>598</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="B37" s="7">
         <v>46083</v>
@@ -6357,64 +6360,64 @@
       <c r="C37" s="1">
         <v>2448</v>
       </c>
-      <c r="D37" s="1" t="s">
-        <v>436</v>
+      <c r="D37" s="9" t="s">
+        <v>636</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>56</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I37" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="P37" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="Q37" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="R37" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="S37" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="T37" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="U37" s="1" t="s">
         <v>441</v>
-      </c>
-      <c r="L37" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="M37" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="P37" s="1" t="s">
-        <v>444</v>
-      </c>
-      <c r="Q37" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="R37" s="1" t="s">
-        <v>608</v>
-      </c>
-      <c r="S37" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="U37" s="1" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="B38" s="7">
         <v>46083</v>
@@ -6423,63 +6426,63 @@
         <v>2449</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>631</v>
+        <v>622</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="O38" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>609</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="H38" s="1" t="s">
+      <c r="P38" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="J38" s="1" t="s">
+      <c r="Q38" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="K38" s="1" t="s">
+      <c r="R38" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="L38" s="1" t="s">
+      <c r="S38" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="M38" s="1" t="s">
+      <c r="T38" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="N38" s="1" t="s">
+      <c r="U38" s="1" t="s">
         <v>456</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="P38" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="Q38" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="R38" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="S38" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="T38" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>464</v>
+        <v>457</v>
       </c>
       <c r="B39" s="7">
         <v>46083</v>
@@ -6488,63 +6491,63 @@
         <v>2451</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>78</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
       <c r="R39" s="1" t="s">
-        <v>610</v>
+        <v>601</v>
       </c>
       <c r="S39" s="1" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="T39" s="1" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="U39" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="B40" s="7">
         <v>46083</v>
@@ -6553,63 +6556,63 @@
         <v>2452</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="P40" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="I40" s="1" t="s">
+      <c r="Q40" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="R40" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="J40" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="K40" s="1" t="s">
+      <c r="S40" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="L40" s="1" t="s">
+      <c r="T40" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="M40" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="N40" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="O40" s="1" t="s">
-        <v>480</v>
-      </c>
-      <c r="P40" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="Q40" s="1" t="s">
-        <v>611</v>
-      </c>
-      <c r="R40" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="S40" s="1" t="s">
-        <v>483</v>
-      </c>
-      <c r="T40" s="1" t="s">
-        <v>484</v>
-      </c>
       <c r="U40" s="1" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
       <c r="B41" s="7">
         <v>46083</v>
@@ -6618,63 +6621,63 @@
         <v>2504</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="L41" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="M41" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>613</v>
-      </c>
-      <c r="G41" s="1" t="s">
+      <c r="N41" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="O41" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="P41" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="Q41" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="R41" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="K41" s="1" t="s">
+      <c r="S41" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="L41" s="1" t="s">
+      <c r="T41" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="M41" s="1" t="s">
+      <c r="U41" s="1" t="s">
         <v>494</v>
-      </c>
-      <c r="N41" s="1" t="s">
-        <v>494</v>
-      </c>
-      <c r="O41" s="1" t="s">
-        <v>495</v>
-      </c>
-      <c r="P41" s="1" t="s">
-        <v>496</v>
-      </c>
-      <c r="Q41" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="R41" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="S41" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="T41" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="U41" s="1" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="B42" s="7">
         <v>46083</v>
@@ -6683,63 +6686,63 @@
         <v>2513</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>614</v>
+        <v>605</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="K42" s="1" t="s">
         <v>104</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>615</v>
+        <v>606</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>616</v>
+        <v>607</v>
       </c>
       <c r="S42" s="1" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
       <c r="U42" s="1" t="s">
-        <v>617</v>
+        <v>608</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
       <c r="B43" s="7">
         <v>46083</v>
@@ -6748,22 +6751,22 @@
         <v>2545</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>31</v>
@@ -6781,30 +6784,30 @@
         <v>31</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="U43" s="1" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="B44" s="7">
         <v>46083</v>
@@ -6813,13 +6816,13 @@
         <v>3682</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>525</v>
+        <v>518</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
@@ -6832,25 +6835,25 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
       <c r="O44" s="1" t="s">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>532</v>
+        <v>525</v>
       </c>
       <c r="U44" s="1" t="s">
-        <v>618</v>
+        <v>609</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revising for symbol formatting
</commit_message>
<xml_diff>
--- a/data/processed/pssi_form_data_altered.xlsx
+++ b/data/processed/pssi_form_data_altered.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\PSSI-final-tech-report\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF8C8F2-6170-4789-9100-586184E57A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCD6B92-F2B7-4073-96DE-24623086BF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="639">
   <si>
     <t>source_file</t>
   </si>
@@ -1042,9 +1042,6 @@
     <t>All freshwater phases</t>
   </si>
   <si>
-    <t>Fraser</t>
-  </si>
-  <si>
     <t>CK-03, CK-04, CK-05, CK-06, CK-07, CK-08, CK-09, CK-10, CK-11, CK-12, CK-14, CK-16, CK-17, CK-18, CK-19, CO-05, CO-07, CO-08, CO-09, CO-48, SEL-03-02, SEL-03-03, SEL-03-04, SEL-04-01, SEL-05-02, SEL-06-07, SEL-06-10, SEL-06-11, SEL-06-13, SEL-06-14, SEL-06-16, SEL-07-01, SEL-09-xx, SEL-10-01, SEL-10-03, SER-02, CK-13, CK-15, CK-82, CM-02, CO-04, CO-47, PKE-9005, PKO-01, SEL-03-01, SEL-03-05, SEL-06-01, SEL-06-02,
 SEL-06-20, SEL-09-02, SEL-09-03, SER-03</t>
   </si>
@@ -1066,10 +1063,6 @@
   <si>
     <t>This project is the first to provide spatially extensive estimates of human activity and climate change threats that are directly linked to salmon, SAR, and their habitats at the stream reach scale. The approaches used to estimate each of the indicators provide an initial broad-scale standardized framework that can be applied to characterize threats throughout the Pacific Region. Within the FRB, we observed the highest threats in the Lower Fraser and interior plateau, and specifically, within the Nicola River, Guichon Creek, and San Jose River. Overall, roads were the greatest contributor to human activity-based threats, disturbing in-stream habitats, riparian areas, and contributing to sediment and nutrient loading. These results improve our understanding of the spatial distribution and relative magnitude of threats across the FRB, providing a foundation for predicting population-level impacts from cumulative effects and life-cycle modelling.
 A major source of uncertainty is the spatial accuracy of the BC Freshwater Atlas. Known issues to the FWA include overestimates of headwater streams in interior regions, misaligned stream delineations and large river catchment areas. Each of the individual threat scores have their own uncertainties and limitations, as detailed in Table 2 of Iacarella et al. (2025). In general, the input data are subject to limitations arising from potentially misclassified land cover or land use, features included in datasets but not present on the landscape, and unmapped activities or features, which introduce uncertainty into individual threat scores and the cumulative score. An additional source of uncertainty is the unresolved habitat use and distribution of salmon and SAR within the FRB. The approach used to combine individual threats into a cumulative threat score (e.g., addition, multiplication, etc.) is another source of uncertainty that can be evaluated in future work by modelling population responses to individual and cumulative threats.</t>
-  </si>
-  <si>
-    <t>Although our threat estimates represent the mechanisms by which salmon and freshwater SAR are affected, the magnitude at which these threats influence salmon population dynamics remains unknown. To address this gap, we are continuing to refine existing threat estimates and developing new threats that are explicitly linked to stressor-response functions for cumulative effects and life-cycle modelling. For example, we have developed additional riparian disturbance metrics that better capture the impacts to riparian function (e.g., large-woody debris recruitment, disturbance to stream-shading, riparian filtering), which were not included in the original report. Moreover, we are developing a stage-structured population model for Interior Fraser Coho (IFC) to estimate how stressors (estimated threats) are influencing the population across their freshwater life stages. For this work, we are utilising the Cumulative Effects Model for Prioritizing Recovery Actions (CEMPRA), which applies stressor-response functions to account for the impact of stressors on vital rates and the overall population overtime and under different climate change and mitigation scenarios (Bayly et al*.* 2024).
-Additional next steps for this work include expanding the cumulative threats model to other watersheds in the Pacific Region. To date, the model has also been applied to the Upper Bulkley Watershed to aid in salmon habitat restoration planning. Validation is an important step of most modelling exercises, though is often not a standard component of cumulative effect assessments (Halpern and Fujita 2013). Validating these threats through field verification and in situ data would be beneficial for threats that involve applied relationships and estimations, such as the flow accumulated loadings (i.e., nutrients, pollution, sedimentation). Future work could re-run the model at regular intervals to evaluate change in threats over time. Finally, additional analyses could quantify uncertainty in modelled threats and evaluate underlying assumptions through sensitivity tests.</t>
   </si>
   <si>
     <t>2426 PSSI Science Project Reporting Template Oct2025_Sakinaw Sockeye_KP-KF.docx</t>
@@ -1570,9 +1563,6 @@
   </si>
   <si>
     <t>Okanagan</t>
-  </si>
-  <si>
-    <t>Canadian Okanagan</t>
   </si>
   <si>
     <t>CK-01</t>
@@ -1604,11 +1594,6 @@
 - using predator-detecting acoustic tags to determine juvenile mortality from predation and finer-scale movement data to elucidate habitat use throughout the migration corridor;
 - estimating the smallmouth bass population size in the Okanagan River and Lake system to quantify the predation pressure on juvenile Chinook; and
 - understanding the role of predation from other native and invasive piscivorous fish and avian predators on juvenile Chinook survival.</t>
-  </si>
-  <si>
-    <t>Figure 1. Proportion of acoustic tagged juvenile Chinook detected at downstream detections sites and resulting survival curves for release Group A (n= 273 upstream of Vaseux Lake) and B (n=274 downstream of McIntyre Dam). In both release groups, there is a sharp decline in the proportion of fish detected and survival is low during the downstream migration.
-Figure 2. DNA metabarcoding stomach content analysis of n=162 smallmouth bass (*Micropterus dolomieu*) captured at various locations in the Okanagan River and Lake system. Aquatic insects (Diptera, Ephemeroptera, Trichoptera), invasive fish (smallmouth bass, yellow perch, common carp), and native fish (prickly sculpin, mountain whitefish, Sockeye/kokanee, Chinook) were the most common prey items identified.
-Table 1. Total length (TL) and weight of the 196 smallmouth bass (*Micropterus dolomieu*) captured in the juvenile Chinook predation study. Bass were captured by angling in the Okanagan River and Lake system and were sacrificed upon capture for stomach content analysis.</t>
   </si>
   <si>
     <t>2443 PSSI Science Project Reporting Template_Project ID.docx</t>
@@ -2757,33 +2742,6 @@
     <t>Chinook Salmon *OncorhynchusÂ tshawytscha*</t>
   </si>
   <si>
-    <t>Low flows during summer months can be an important bottleneck for stream-rearing rearing salmon. Determining how much water fish need is therefore a critical management question, especially given rising human water use and climate warming. Elevated water temperature is another threat facing stream-rearing salmon that is often linked to low flows. However, conventional modelling tools for determining instream flow needs have generally not explicitly considered temperature. This is a gap for management as it is unclear if current instream flow assessments will apply in a warmer future.
-This project developed an analytical framework to integrate water temperature into habitat simulation models, a widely used tool for determining instream flow needs. We used a bioenergetics framework that relates channel hydraulics (e.g., depth and velocity) and temperature to the daily energy balance of juvenile salmonids. We then applied the approach to 17 coho-rearing streams across the North Thompson watershed, interior BC. This work was collaborative with SecwÃ©pemc Fisheries Commission and Simpcw First Nation and will inform instream flow management through the lens of climate change.</t>
-  </si>
-  <si>
-    <t>We used a habitat simulation model framework that links streamflow to channel hydraulics, then channel hydraulics to fish using bioenergetics. The end result is a matrix of relative habitat availability across combinations of flow and water temperature. This can be used as a tool to support real-time flow and temperature monitoring or be linked to flow and temperature projections under contrasting climate change scenarios. Initial model outputs have been shared with SecwÃ©pemc Fisheries Commission to support drought monitoring in several priority systems.
-Flow-habitat relationships were variable across the different streams, suggesting that generic thresholds of flow (e.g., 20% of mean annual discharge) may not always apply. The combined effect of flow and temperature was also variable, reflecting the complex nonlinear pathways that temperature influences fish.
-While the specific model outputs generated to date are applicable to the North Thompson, the general approach is broadly applicable to other systems where the combined impacts of flow and temperature change are of interest.</t>
-  </si>
-  <si>
-    <t>Railsback, S.F., 2016. Why it is time to put PHABSIM out to pasture.Â *Fisheries*,Â *41*(12), pp.720-725.
-Naman, S.M., Rosenfeld, J.S., Neuswanger, J.R., Enders, E.C., Hayes, J.W., Goodwin, E.O., Jowett, I.G. and Eaton, B.C., 2020. Bioenergetic Habitat Suitability Curves for Instream Flow Modeling: Introducing Userâ€Friendly Software and its Potential Applications.Â *Fisheries*,Â *45*(11), pp.605-613.</t>
-  </si>
-  <si>
-    <t>Figure 1. (a) Human activity and landscape disturbance based additive cumulative threat score, and (b) Climate change additive cumulative threat score for 2040-2060 under RCP 4.5. Blue indicates low threat levels and red indicates high threat levels.
-Figure 2. Tukey's box-whiskers plots of the cumulative threat scores from human activity and landscape disturbance based threats and climate change based threats for all streams in the FRB, (a &amp; b) accessible streams within salmon CUs, and (c &amp; d) delineated stream habitats of fish SAR. Salmon CUs identified as Special Concern, Threatened, or Endangered by COSEWIC were distinguished from those not at risk.
-Figure 3. Median cumulative threat composite scores for watershed groups in the Thompson-Nicola EDU based on the multiplicative value of human activity and landscape disturbance based cumulative threats and modeled environmental favourability for spawning (row a) Chinook, (b) Coho, (c) Pink, and (d) Sockeye Salmon. Modeled environmental favourability probabilities used in the composite score were based on projected (column a) current and (b) future conditions for all stream reaches (â‰¥ 4th order) including inaccessible streams from dams and natural barriers. Watershed groups that are largely inaccessible are identified by hatched lines, and salmon CU boundaries in black outlines. Colour scale indicates increasing need for localized investigation and potential restoration.</t>
-  </si>
-  <si>
-    <t>Bayly, M., Tekatch, A., Rosenfeld, J., Jarvis, L. &amp; Enders, E. 2024. Cumulative Effects Model for Prioritizing Recovery Actions (CEMPRA): User Guide. Documentation prepared by ESSA Technologies Ltd. for the BC Water, Land and Resource S. Available from: https://essatech.github.io/CEMPRA/ [accessed 29 December 2025].
-DFO. 2022. Geospatial mapping tools, indicators, and metrics for fish habitat in the Pacific Region. DFO Can. Sci. Advis. Sec. Sci. Resp. 2022/047.
-Halpern, B.S., and Fujita, R. 2013. Assumptions, challenges, and future directions in cumulative impact analysis. Ecosphere. 4: art131. doi:10.1890/ES13-00181.1
-Halpern, B.S., McLeod, K.L., Rosenberg, A.A., and Crowder, L.B. 2008a. Managing for cumulative impacts in ecosystem-based management through ocean zoning. Ocean Coast. Manage. 51: 203-211. doi:10.1016/j.ocecoaman.2007.08.002
-Iacarella, J.C. and Weller, J.D., 2023. Predicting favourable streams for anadromous salmon spawning and natal rearing under climate change.Â Can. J. Fish. Aquat. Sci.,Â 81(1), pp.1-13. doi:10.1139/cjfas-2023-0096
-Iacarella, J.C., Paterson, K., Potapova, A., and Weller, J.D. 2025. Geospatial Indicators and Metrics for Threats to Fish Habitat in the Fraser River Basin with Thompson-Nicola as a Case Study. DFO Can. Sci. Advis. Sec. Res. Doc. 2025/013. xiii + 126 p.
-Rosenfeld, J., Gonzalez-Espinosa, P., Jarvis, L., Enders, E., Bayly, M., Paul, A., MacPherson, L., Moore, J., Sullivan, M., Ulaski, M., and Wilson, K. 2022. Stressor-response functions as a generalizable model for context dependence. Trends Ecol. Evolut. 37: 1032-1035. doi:10.1016/j.tree.2022.09.010</t>
-  </si>
-  <si>
     <t>Sakinaw sockeye have been listed as endangered with COSEWIC since 2003, and a *Species at Risk Act* Recovery Potential Assessment (RPA) was completed in 2017 (Ramshaw et al. 2019). The RPA cited low marine survival as the greatest limiting factor in recovery, with predator abundance and assumed predation on smolts and adults ranked as high risk, with a critical level of impact. Perpetually low marine survivals are preventing recovery such that the persistence of the population is entirely dependent on a captive brood program.
 Sakinaw sockeye smolts out-migrate from Sakinaw Lake each spring into the Malaspina Strait and Strait of Georgia. Localized marine predation is considered a major limiting factor for the survival of this stock. On water surveys (since 2019) of pinnipeds from the estuary to the seal haul-outs on Hodgson Islands (approximately 2km from the estuary, Figure 1) have observed approximately 100-350 harbour seals in the area during the spring out-migration.
 This project was started as a pilot (2022) in collaboration with shÃ­shÃ¡lh Nation to test the hypothesis that the Hodgson Island harbour seal population is negatively affecting smolt survival, and subsequently adult returns. The goal of the project is to transport and release smolts past the seal haul-out and then compare marine survival rates between transported smolts and those out-migrating naturally. The pilot project began with a low number of smolts transported in small trial releases to test the effect of handling, Passive Integrated Transponders (PIT) tagging, and increased osmoregulation on fish.
@@ -3197,16 +3155,54 @@
 Foreman, M.G.G., Chandler, P.C., Bianucci, L., Wan, D., Krassovski, M.V., Thupaki, P., Cooper, G. and Lin, Y., 2024. A circulation model for inlets along the central West Coast of Vancouver Island. Atmosphere-Ocean, 62(1), pp.58-89.</t>
   </si>
   <si>
-    <t xml:space="preserve">Habitat use and survival
-Subyearling Chinook (n=547) raised in the kł cp̓əlk̓ stim̓ hatchery were implanted with ATS SS400 injectable acoustic transmitters. They were released in two groups, with group A (n=273) released in the Okanagan River below Vertical Drop Structure (VDS) 17 and above Vaseux Lake, and group B (n=274) released downstream of Vaseux lake below McIntyre Dam. A network of 15 ATS SR3001 autonomous receivers was deployed from Okanagan Falls to Osoyoos Lake between 21 May and 8 August, 2024). Receivers were clustered into 7 detection sites, placed to form acoustic “gates” at lake inlets and outlets, narrows and channel constrictions, and potential rearing/migration corridors. An ATS SR3017 mobile receiver with hydrophone was used to survey shallow side channels, deeper offshore areas beyond stationary coverage, and upstream and downstream of VDS structures. The proportion of fish detected decreased sharply for both release groups as fish migrated downstream, which translated to low survival in both release groups. Tag burden was not deemed a source of direct mortality, but could have increased susceptibility to predation. 
-Smallmouth bass diet and predation
-Targeted angling was conducted in the Okanagan River, Vaseux Lake, Osoyoos Lake from May 3 to August 7, 2024. The dominant species captured were smallmouth bass, which comprised 76% of the total catch (n=196), followed by Northern Pikeminnow (16%, n=41) and Yellow Perch (4%, n=11). There was a spatial shift in the distribution of smallmouth bass caught during the study. In May, less than half (45%) of smallmouth bass were caught at Vertical Drop Structures (VDS), but the proportion of smallmouth bass captured at VDS structures increased to 100% and 80% in June and July, respectively. Bass were observed utilizing rocky substrate and rip rap below the VDS structures to ambush prey. Diet content visual analysis was performed on a subsample of 73 of the total 196 smallmouth bass. A total of 162 fish stomach samples were sent for DNA barcode sequencing. Chinook salmon was only detected once in the DNA samples, but direct evidence of bass predation on juvenile Chinook was obtained by recovery of an acoustic tag used in the juvenile migration and habitat use study. DNA metabarcoding identified a diverse assemblage of 146 unique prey taxa. Aquatic insects (Diptera,  Ephemeroptera, Trichoptera), invasive fish (smallmouth bass, yellow perch, common carp), and native fish (prickly sculpin, mountain whitefish, sockeye/kokanee, Chinook) were the most common prey items in smallmouth bass stomach contents. </t>
-  </si>
-  <si>
     <t>Electrofishing and angling was conducted in the spring to target SMB as they move to near-shore habitat to build nests and spawn. The perimeter of Cultus Lake was divided into quadrants (Figure 1) and swept with a boat electrofishing unit to target spawning SMB. In 2023, ten consecutive days of electrofishing were conducted (June 1-10, 2023), and all SMB captured (by electrofishing and angling) were implanted with a PIT tag and released to get an initial baseline of the population in 2024. A subset of SMB (n=25) were also implanted with acoustic transmitters to track movements within the lake, and downstream movement from the lake (acoustic receivers also deployed in 2023 in various locations). In 2024, two consecutive days (east side of lake day one; west side of lake day two) of electrofishing and angling were conducted for six consecutive weeks (May 9 - June 7, 2024), and all SMB were euthanized to get a PIT tag recovery sample and to see how the population responded to the cull the following year. In 2025, operations were conducted in two day intervals, for seven consecutive weeks (May 1 - June 13, 2025). For the first two weeks of the project all SMB were euthanized to reduce the spawning potential of the population, and for subsequent weeks 25% of all SMB were implanted with PIT tags and released. A subset of 44 SMB were also implanted with acoustic transmitters to track movements within, and from Cultus Lake. A total of 3,654 biological samples (length, weight (Figure 2); subset of stomach contents (Figure 3), scales, otoliths) were collected from SMB between 2023-2025. Of these samples, 268 stomach samples, 2,069 scale samples, and 20 otoliths samples were collected. Age analysis and acoustic tracking results are pending, and will be included in the final report (written by SFU).
 Between 2023 and 2025, a total of 6,650 SMB were captured by a combination of electrofishing and angling (942 in 2023, 1,616 in 2024, 4,092 in 2025; 95% by electrofishing, 5% by angling). A total of 1,469 PIT tags were deployed (897 in 2023, 572 in 2025), and 69 acoustic tags were surgically implanted in SMB (25 in 2023, 44 in 2025). Of the PIT tags deployed in 2023, 47 were recaptured in 2024 (4.8% recovery) and 12 were recaptured in 2025 (1.2% recovery), giving a rough population estimate of approximately 16,000 SMB in 2024. However, observations from staff at the Cultus Lake Laboratory, the Province of BC, and anglers have indicated a significant portion of the population occupy habitat at depths that preclude SMB from capture by electrofishing, thus, this estimate is likely biased low. The PIT tags deployed in 2025 have yet to be captured in 2026, therefore a current population estimate is unavailable at this time. It should be noted that in 2023, a total of two pumpkinseed were captured during the electrofishing program. In 2024 the number increased to 60, and in 2025 increased to 2,553. Further to this, the capture of pumpkinseed was incidental as there is some overlap in habitat with SMB, and if efforts were targeted for pumpkinseed (i.e. heavily vegetated near-shore habitat), those numbers would be higher. The rapid increase in pumpkinseed bycatch over the course of this work is alarming and should be investigated in future years.
 The subset of stomach samples taken, approximately 10% of samples contained juvenile salmonids (fry or smolt stage), and 2% contained sculpins. It is noted that many stomach samples were at an advanced stage of digestion therefore these estimates are biased low. Acoustic tracking of SMB is ongoing and will be discussed in the final report. However, between 2024 and 2025 a total of 17 SMB were captured at the DFO-operated smolt enumeration fence (run March - June annually), indicating some downstream movement of SMB in Sweltzer Creek to the Vedder River (tributary to the Fraser River). At this time there are no confirmed reports of SMB in the Vedder or Fraser rivers, however, as the population in Cultus Lake expands, downstream colonization is likely.
 The following results, in addition to acoustic tracking data, an evaluation of suppression methods (paired with feedback from the public and social survey results), and up-to-date SMB population estimates will be presented in the final report written by SFU, DFO and the Province of BC in 2027.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Habitat use and survival*
+Subyearling Chinook (n=547) raised in the kł cp̓əlk̓ stim̓ hatchery were implanted with ATS SS400 injectable acoustic transmitters. They were released in two groups, with group A (n=273) released in the Okanagan River below Vertical Drop Structure (VDS) 17 and above Vaseux Lake, and group B (n=274) released downstream of Vaseux lake below McIntyre Dam. A network of 15 ATS SR3001 autonomous receivers was deployed from Okanagan Falls to Osoyoos Lake between 21 May and 8 August, 2024). Receivers were clustered into 7 detection sites, placed to form acoustic “gates” at lake inlets and outlets, narrows and channel constrictions, and potential rearing/migration corridors. An ATS SR3017 mobile receiver with hydrophone was used to survey shallow side channels, deeper offshore areas beyond stationary coverage, and upstream and downstream of VDS structures. The proportion of fish detected decreased sharply for both release groups as fish migrated downstream, which translated to low survival in both release groups. Tag burden was not deemed a source of direct mortality, but could have increased susceptibility to predation. 
+*Smallmouth bass diet and predation*
+Targeted angling was conducted in the Okanagan River, Vaseux Lake, Osoyoos Lake from May 3 to August 7, 2024. The dominant species captured were smallmouth bass, which comprised 76% of the total catch (n=196), followed by Northern Pikeminnow (16%, n=41) and Yellow Perch (4%, n=11). There was a spatial shift in the distribution of smallmouth bass caught during the study. In May, less than half (45%) of smallmouth bass were caught at Vertical Drop Structures (VDS), but the proportion of smallmouth bass captured at VDS structures increased to 100% and 80% in June and July, respectively. Bass were observed utilizing rocky substrate and rip rap below the VDS structures to ambush prey. Diet content visual analysis was performed on a subsample of 73 of the total 196 smallmouth bass. A total of 162 fish stomach samples were sent for DNA barcode sequencing. Chinook salmon was only detected once in the DNA samples, but direct evidence of bass predation on juvenile Chinook was obtained by recovery of an acoustic tag used in the juvenile migration and habitat use study. DNA metabarcoding identified a diverse assemblage of 146 unique prey taxa. Aquatic insects (Diptera,  Ephemeroptera, Trichoptera), invasive fish (smallmouth bass, yellow perch, common carp), and native fish (prickly sculpin, mountain whitefish, sockeye/kokanee, Chinook) were the most common prey items in smallmouth bass stomach contents. </t>
+  </si>
+  <si>
+    <t>Low flows during summer months can be an important bottleneck for stream-rearing rearing salmon. Determining how much water fish need is therefore a critical management question, especially given rising human water use and climate warming. Elevated water temperature is another threat facing stream-rearing salmon that is often linked to low flows. However, conventional modelling tools for determining instream flow needs have generally not explicitly considered temperature. This is a gap for management as it is unclear if current instream flow assessments will apply in a warmer future. 
+This project developed an analytical framework to integrate water temperature into habitat simulation models, a widely used tool for determining instream flow needs. We used a bioenergetics framework that relates channel hydraulics (e.g., depth and velocity) and temperature to the daily energy balance of juvenile salmonids. We then applied the approach to 17 coho-rearing streams across the North Thompson watershed, interior BC. This work was collaborative with Secwépemc Fisheries Commission and Simpcw First Nation and will inform instream flow management through the lens of climate change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We used a habitat simulation model framework that links streamflow to channel hydraulics, then channel hydraulics to fish using bioenergetics. The end result is a matrix of relative habitat availability across combinations of flow and water temperature. This can be used as a tool to support real-time flow and temperature monitoring or be linked to flow and temperature projections under contrasting climate change scenarios. Initial model outputs have been shared with Secwépemc Fisheries Commission to support drought monitoring in several priority systems. 
+Flow-habitat relationships were variable across the different streams, suggesting that generic thresholds of flow (e.g., 20% of mean annual discharge) may not always apply. The combined effect of flow and temperature was also variable, reflecting the complex nonlinear pathways that temperature influences fish. 
+While the specific model outputs generated to date are applicable to the North Thompson, the general approach is broadly applicable to other systems where the combined impacts of flow and temperature change are of interest. </t>
+  </si>
+  <si>
+    <t>Railsback, S.F., 2016. Why it is time to put PHABSIM out to pasture. Fisheries, 41(12), pp.720-725.
+Naman, S.M., Rosenfeld, J.S., Neuswanger, J.R., Enders, E.C., Hayes, J.W., Goodwin, E.O., Jowett, I.G. and Eaton, B.C., 2020. Bioenergetic Habitat Suitability Curves for Instream Flow Modeling: Introducing User‐Friendly Software and its Potential Applications. Fisheries, 45(11), pp.605-613.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 1. (a) Human activity and landscape disturbance based additive cumulative threat score, and (b) Climate change additive cumulative threat score for 2040-2060 under RCP 4.5. Blue indicates low threat levels and red indicates high threat levels.
+Figure 2. Tukey’s box-whiskers plots of the cumulative threat scores from human activity and landscape disturbance based threats and climate change based threats for all streams in the FRB, (a &amp; b) accessible streams within salmon CUs, and (c &amp; d) delineated stream habitats of fish SAR. Salmon CUs identified as Special Concern, Threatened, or Endangered by COSEWIC were distinguished from those not at risk. 
+Figure 3. Median cumulative threat composite scores for watershed groups in the Thompson-Nicola EDU based on the multiplicative value of human activity and landscape disturbance based cumulative threats and modeled environmental favourability for spawning (row a) Chinook, (b) Coho, (c) Pink, and (d) Sockeye Salmon. Modeled environmental favourability probabilities used in the composite score were based on projected (column a) current and (b) future conditions for all stream reaches (≥ 4th order) including inaccessible streams from dams and natural barriers. Watershed groups that are largely inaccessible are identified by hatched lines, and salmon CU boundaries in black outlines. Colour scale indicates increasing need for localized investigation and potential restoration. </t>
+  </si>
+  <si>
+    <t>Although our threat estimates represent the mechanisms by which salmon and freshwater SAR are affected, the magnitude at which these threats influence salmon population dynamics remains unknown. To address this gap, we are continuing to refine existing threat estimates and developing new threats that are explicitly linked to stressor-response functions for cumulative effects and life-cycle modelling. For example, we have developed additional riparian disturbance metrics that better capture the impacts to riparian function (e.g., large-woody debris recruitment, disturbance to stream-shading, riparian filtering), which were not included in the original report. Moreover, we are developing a stage-structured population model for Interior Fraser Coho (IFC) to estimate how stressors (estimated threats) are influencing the population across their freshwater life stages. For this work, we are utilizing the Cumulative Effects Model for Prioritizing Recovery Actions (CEMPRA), which applies stressor-response functions to account for the impact of stressors on vital rates and the overall population overtime and under different climate change and mitigation scenarios (Bayly et al. 2024).
+Additional next steps for this work include expanding the cumulative threats model to other watersheds in the Pacific Region. To date, the model has also been applied to the Upper Bulkley Watershed to aid in salmon habitat restoration planning. Validation is an important step of most modelling exercises, though is often not a standard component of cumulative effect assessments (Halpern and Fujita 2013). Validating these threats through field verification and in situ data would be beneficial for threats that involve applied relationships and estimations, such as the flow accumulated loadings (i.e., nutrients, pollution, sedimentation). Future work could re-run the model at regular intervals to evaluate change in threats over time. Finally, additional analyses could quantify uncertainty in modelled threats and evaluate underlying assumptions through sensitivity tests.</t>
+  </si>
+  <si>
+    <t>Bayly, M., Tekatch, A., Rosenfeld, J., Jarvis, L. &amp; Enders, E. 2024. Cumulative Effects Model for Prioritizing Recovery Actions (CEMPRA): User Guide. Documentation prepared by ESSA Technologies Ltd. for the BC Water, Land and Resource S. Available from: https://essatech.github.io/CEMPRA/ [accessed 29 December 2025].
+DFO. 2022. Geospatial mapping tools, indicators, and metrics for fish habitat in the Pacific Region. DFO Can. Sci. Advis. Sec. Sci. Resp. 2022/047. 
+Halpern, B.S., and Fujita, R. 2013. Assumptions, challenges, and future directions in cumulative impact analysis. Ecosphere. 4: art131. doi:10.1890/ES13-00181.1
+Halpern, B.S., McLeod, K.L., Rosenberg, A.A., and Crowder, L.B. 2008a. Managing for cumulative impacts in ecosystem-based management through ocean zoning. Ocean Coast. Manage. 51: 203–211. doi:10.1016/j.ocecoaman.2007.08.002		 
+Iacarella, J.C. and Weller, J.D., 2023. Predicting favourable streams for anadromous salmon spawning and natal rearing under climate change. Can. J. Fish. Aquat. Sci., 81(1), pp.1-13. doi:10.1139/cjfas-2023-0096
+Iacarella, J.C., Paterson, K., Potapova, A., and Weller, J.D. 2025. Geospatial Indicators and Metrics for Threats to Fish Habitat in the Fraser River Basin with Thompson-Nicola as a Case Study. DFO Can. Sci. Advis. Sec. Res. Doc. 2025/013. xiii + 126 p.
+Rosenfeld, J., Gonzalez-Espinosa, P., Jarvis, L., Enders, E., Bayly, M., Paul, A., MacPherson, L., Moore, J., Sullivan, M., Ulaski, M., and Wilson, K. 2022. Stressor-response functions as a generalizable model  for context dependence. Trends Ecol. Evolut. 37: 1032–1035.   doi:10.1016/j.tree.2022.09.010
+Iacarella, J.C., Paterson, K., Potapova, A., and Weller, J.D. 2025. Geospatial Indicators and Metrics for Threats to Fish Habitat in the Fraser River Basin with Thompson-Nicola as a Case Study. DFO Can. Sci. Advis. Sec. Res. Doc. 2025/013. xiii + 126 p.
+Rosenfeld, J., Gonzalez-Espinosa, P., Jarvis, L., Enders, E., Bayly, M., Paul, A., MacPherson, L., Moore, J., Sullivan, M., Ulaski, M., and Wilson, K. 2022. Stressor-response functions as a generalizable model for context dependence. Trends Ecol. Evolut. 37: 1032-1035. doi:10.1016/j.tree.2022.09.010</t>
+  </si>
+  <si>
+    <t>Figure 1. Proportion of acoustic tagged juvenile Chinook detected at downstream detections sites and resulting survival curves for release Group A (n= 273 upstream of Vaseux Lake) and B (n=274 downstream of McIntyre Dam). In both release groups, there is a sharp decline in the proportion of fish detected and survival is low during the downstream migration.
+Figure 2. DNA metabarcoding stomach content analysis of n=162 smallmouth bass (*Micropterus dolomieu*) captured at various locations in the Okanagan River and Lake system. Aquatic insects (Diptera, Ephemeroptera, Trichoptera), invasive fish (smallmouth bass, yellow perch, common carp), and native fish (prickly sculpin, mountain whitefish, sockeye/kokanee, Chinook) were the most common prey items identified.
+Table 1. Total length (TL) and weight of the 196 smallmouth bass (*Micropterus dolomieu*) captured in the juvenile Chinook predation study. Bass were captured by angling in the Okanagan River and Lake system and were sacrificed upon capture for stomach content analysis.</t>
   </si>
 </sst>
 </file>
@@ -4104,7 +4100,7 @@
         <v>22</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -4134,7 +4130,7 @@
         <v>31</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>32</v>
@@ -4184,7 +4180,7 @@
         <v>44</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>45</v>
@@ -4193,13 +4189,13 @@
         <v>46</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>47</v>
@@ -4234,13 +4230,13 @@
         <v>2400</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>635</v>
+        <v>626</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>56</v>
@@ -4249,7 +4245,7 @@
         <v>57</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>58</v>
@@ -4261,19 +4257,19 @@
         <v>59</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="P4" s="1" t="s">
         <v>60</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
       <c r="R4" s="1" t="s">
         <v>61</v>
@@ -4282,10 +4278,10 @@
         <v>62</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -4299,16 +4295,16 @@
         <v>2401</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>64</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>65</v>
@@ -4340,7 +4336,7 @@
         <v>72</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
@@ -4381,7 +4377,7 @@
         <v>81</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>82</v>
@@ -4393,7 +4389,7 @@
         <v>84</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>85</v>
@@ -4419,7 +4415,7 @@
         <v>2403</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>90</v>
@@ -4440,7 +4436,7 @@
         <v>95</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="L7" s="4" t="s">
         <v>96</v>
@@ -4449,7 +4445,7 @@
         <v>96</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>613</v>
+        <v>604</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>97</v>
@@ -4458,19 +4454,19 @@
         <v>98</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>614</v>
+        <v>605</v>
       </c>
       <c r="T7" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="U7" s="4" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
     </row>
     <row r="8" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4490,31 +4486,31 @@
         <v>101</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>102</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>103</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>104</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O8" s="4" t="s">
         <v>105</v>
@@ -4523,7 +4519,7 @@
         <v>106</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="R8" s="4" t="s">
         <v>107</v>
@@ -4532,10 +4528,10 @@
         <v>108</v>
       </c>
       <c r="T8" s="4" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>638</v>
+        <v>629</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
@@ -4552,19 +4548,19 @@
         <v>110</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>621</v>
+        <v>612</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>111</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>112</v>
@@ -4573,13 +4569,13 @@
         <v>113</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>114</v>
@@ -4588,7 +4584,7 @@
         <v>115</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="R9" s="1" t="s">
         <v>116</v>
@@ -4600,7 +4596,7 @@
         <v>118</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
@@ -4620,40 +4616,40 @@
         <v>121</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>122</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>124</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>125</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="R10" s="1" t="s">
         <v>126</v>
@@ -4679,13 +4675,13 @@
         <v>2407</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>636</v>
+        <v>627</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>131</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>623</v>
+        <v>614</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>132</v>
@@ -4703,10 +4699,10 @@
         <v>56</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N11" s="4" t="s">
         <v>136</v>
@@ -4727,10 +4723,10 @@
         <v>141</v>
       </c>
       <c r="T11" s="4" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
       <c r="U11" s="4" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
@@ -4744,13 +4740,13 @@
         <v>2408</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>56</v>
@@ -4777,7 +4773,7 @@
         <v>146</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="R12" s="1" t="s">
         <v>147</v>
@@ -4786,10 +4782,10 @@
         <v>148</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
@@ -4828,7 +4824,7 @@
         <v>156</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>157</v>
@@ -4849,10 +4845,10 @@
         <v>162</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -4872,31 +4868,31 @@
         <v>165</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>31</v>
+        <v>522</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>522</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>31</v>
+      <c r="J14" s="9" t="s">
+        <v>522</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L14" s="1" t="s">
-        <v>31</v>
+      <c r="L14" s="9" t="s">
+        <v>522</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>31</v>
+        <v>522</v>
+      </c>
+      <c r="N14" s="9" t="s">
+        <v>522</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>167</v>
@@ -4917,7 +4913,7 @@
         <v>172</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>637</v>
+        <v>628</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
@@ -4931,7 +4927,7 @@
         <v>2412</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>618</v>
+        <v>609</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>174</v>
@@ -4943,34 +4939,34 @@
         <v>176</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>177</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>56</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>178</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="R15" s="1" t="s">
         <v>179</v>
@@ -4979,10 +4975,10 @@
         <v>180</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -4996,13 +4992,13 @@
         <v>2413</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>629</v>
+        <v>620</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>182</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>183</v>
@@ -5020,13 +5016,13 @@
         <v>186</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O16" s="1" t="s">
         <v>187</v>
@@ -5044,7 +5040,7 @@
         <v>191</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="U16" s="1" t="s">
         <v>192</v>
@@ -5067,7 +5063,7 @@
         <v>195</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>196</v>
@@ -5091,10 +5087,10 @@
         <v>104</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="P17" s="1" t="s">
         <v>201</v>
@@ -5141,7 +5137,7 @@
         <v>212</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>213</v>
@@ -5153,10 +5149,10 @@
         <v>215</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>216</v>
@@ -5165,19 +5161,19 @@
         <v>217</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="S18" s="1" t="s">
         <v>218</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="U18" s="1" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -5191,13 +5187,13 @@
         <v>2418</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>630</v>
+        <v>621</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>209</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>220</v>
@@ -5206,7 +5202,7 @@
         <v>221</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>222</v>
@@ -5218,31 +5214,31 @@
         <v>223</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>224</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="S19" s="1" t="s">
         <v>225</v>
       </c>
       <c r="T19" s="5" t="s">
-        <v>615</v>
+        <v>606</v>
       </c>
       <c r="U19" s="1" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -5256,22 +5252,22 @@
         <v>2421</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>631</v>
+        <v>622</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>227</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>197</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>228</v>
@@ -5280,13 +5276,13 @@
         <v>56</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>229</v>
@@ -5295,7 +5291,7 @@
         <v>230</v>
       </c>
       <c r="Q20" s="1" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="R20" s="1" t="s">
         <v>231</v>
@@ -5304,10 +5300,10 @@
         <v>232</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="U20" s="1" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
@@ -5327,13 +5323,13 @@
         <v>235</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>196</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>236</v>
@@ -5348,10 +5344,10 @@
         <v>238</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O21" s="1" t="s">
         <v>239</v>
@@ -5372,7 +5368,7 @@
         <v>244</v>
       </c>
       <c r="U21" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
@@ -5392,10 +5388,10 @@
         <v>247</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>248</v>
@@ -5410,22 +5406,22 @@
         <v>251</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="P22" s="1" t="s">
-        <v>571</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>572</v>
+      <c r="P22" s="5" t="s">
+        <v>632</v>
+      </c>
+      <c r="Q22" s="5" t="s">
+        <v>633</v>
       </c>
       <c r="R22" s="1" t="s">
         <v>253</v>
@@ -5436,8 +5432,8 @@
       <c r="T22" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="U22" s="1" t="s">
-        <v>573</v>
+      <c r="U22" s="5" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -5451,13 +5447,13 @@
         <v>2425</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>257</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>258</v>
@@ -5471,43 +5467,43 @@
       <c r="J23" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="K23" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N23" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="L23" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N23" s="1" t="s">
+      <c r="O23" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="O23" s="1" t="s">
+      <c r="P23" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="P23" s="1" t="s">
+      <c r="Q23" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="Q23" s="1" t="s">
+      <c r="R23" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="R23" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="S23" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>574</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>575</v>
+      <c r="S23" s="5" t="s">
+        <v>636</v>
+      </c>
+      <c r="T23" s="5" t="s">
+        <v>635</v>
+      </c>
+      <c r="U23" s="5" t="s">
+        <v>637</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B24" s="7">
         <v>46083</v>
@@ -5516,63 +5512,63 @@
         <v>2426</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>617</v>
+        <v>608</v>
       </c>
       <c r="E24" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>607</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="F24" s="9" t="s">
-        <v>616</v>
-      </c>
-      <c r="G24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="L24" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="M24" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="L24" s="1" t="s">
+      <c r="N24" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="M24" s="1" t="s">
+      <c r="O24" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="N24" s="1" t="s">
+      <c r="P24" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="R24" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="O24" s="1" t="s">
+      <c r="S24" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="P24" s="1" t="s">
-        <v>576</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>577</v>
-      </c>
-      <c r="R24" s="1" t="s">
+      <c r="T24" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="S24" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>281</v>
-      </c>
       <c r="U24" s="1" t="s">
-        <v>578</v>
+        <v>569</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B25" s="7">
         <v>46083</v>
@@ -5581,63 +5577,63 @@
         <v>2427</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>182</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>177</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="O25" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="P25" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="L25" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="O25" s="1" t="s">
+      <c r="Q25" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="R25" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="P25" s="1" t="s">
+      <c r="S25" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="Q25" s="1" t="s">
-        <v>579</v>
-      </c>
-      <c r="R25" s="1" t="s">
+      <c r="T25" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="S25" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>291</v>
-      </c>
       <c r="U25" s="1" t="s">
-        <v>580</v>
+        <v>571</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B26" s="7">
         <v>46083</v>
@@ -5646,63 +5642,63 @@
         <v>2430</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>608</v>
+        <v>599</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="J26" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>581</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="L26" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="M26" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N26" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="L26" s="1" t="s">
+      <c r="O26" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="M26" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N26" s="1" t="s">
+      <c r="P26" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="S26" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="O26" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>609</v>
-      </c>
-      <c r="Q26" s="1" t="s">
-        <v>582</v>
-      </c>
-      <c r="R26" s="1" t="s">
-        <v>610</v>
-      </c>
-      <c r="S26" s="1" t="s">
-        <v>300</v>
-      </c>
       <c r="T26" s="1" t="s">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="U26" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B27" s="7">
         <v>46083</v>
@@ -5711,22 +5707,22 @@
         <v>2432</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>622</v>
+        <v>613</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>583</v>
+        <v>574</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>250</v>
@@ -5735,39 +5731,39 @@
         <v>186</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O27" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="P27" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q27" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="P27" s="1" t="s">
+      <c r="R27" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="Q27" s="1" t="s">
+      <c r="S27" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="R27" s="1" t="s">
+      <c r="T27" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="S27" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="T27" s="1" t="s">
-        <v>309</v>
-      </c>
       <c r="U27" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B28" s="7">
         <v>46083</v>
@@ -5776,63 +5772,63 @@
         <v>2433</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>613</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="G28" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="E28" s="9" t="s">
-        <v>622</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>313</v>
-      </c>
       <c r="H28" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>250</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>584</v>
+        <v>575</v>
       </c>
       <c r="P28" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="R28" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="Q28" s="1" t="s">
+      <c r="S28" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="R28" s="1" t="s">
+      <c r="T28" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="S28" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="T28" s="1" t="s">
-        <v>318</v>
-      </c>
       <c r="U28" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B29" s="7">
         <v>46083</v>
@@ -5841,63 +5837,63 @@
         <v>2434</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>323</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>197</v>
       </c>
       <c r="I29" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="L29" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="M29" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="L29" s="1" t="s">
+      <c r="N29" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="M29" s="1" t="s">
+      <c r="O29" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="P29" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="N29" s="1" t="s">
+      <c r="Q29" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="O29" s="1" t="s">
-        <v>585</v>
-      </c>
-      <c r="P29" s="1" t="s">
+      <c r="R29" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="Q29" s="1" t="s">
+      <c r="S29" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="R29" s="1" t="s">
+      <c r="T29" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="S29" s="1" t="s">
+      <c r="U29" s="1" t="s">
         <v>332</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="U29" s="1" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B30" s="7">
         <v>46083</v>
@@ -5906,63 +5902,63 @@
         <v>2435</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>619</v>
+        <v>610</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="J30" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="K30" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="L30" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="M30" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="L30" s="1" t="s">
+      <c r="N30" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="M30" s="1" t="s">
+      <c r="O30" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="N30" s="1" t="s">
+      <c r="P30" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="O30" s="1" t="s">
+      <c r="Q30" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="P30" s="1" t="s">
+      <c r="R30" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="Q30" s="1" t="s">
+      <c r="S30" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="R30" s="1" t="s">
+      <c r="T30" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="S30" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>351</v>
-      </c>
       <c r="U30" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B31" s="7">
         <v>46083</v>
@@ -5971,63 +5967,63 @@
         <v>2436</v>
       </c>
       <c r="D31" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="G31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="J31" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="I31" s="1" t="s">
+      <c r="K31" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="L31" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N31" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="K31" s="1" t="s">
+      <c r="O31" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="L31" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N31" s="1" t="s">
+      <c r="P31" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="O31" s="1" t="s">
+      <c r="Q31" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="P31" s="1" t="s">
+      <c r="R31" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="Q31" s="1" t="s">
+      <c r="S31" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="R31" s="1" t="s">
+      <c r="T31" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="S31" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="T31" s="1" t="s">
-        <v>366</v>
-      </c>
       <c r="U31" s="1" t="s">
-        <v>586</v>
+        <v>577</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B32" s="7">
         <v>46083</v>
@@ -6036,63 +6032,63 @@
         <v>2437</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="H32" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="I32" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="F32" s="1" t="s">
-        <v>587</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="H32" s="1" t="s">
+      <c r="J32" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="I32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="L32" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="M32" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="L32" s="1" t="s">
+      <c r="N32" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="M32" s="1" t="s">
+      <c r="O32" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="P32" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="N32" s="1" t="s">
+      <c r="Q32" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="O32" s="1" t="s">
-        <v>588</v>
-      </c>
-      <c r="P32" s="1" t="s">
+      <c r="R32" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="Q32" s="1" t="s">
+      <c r="S32" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="R32" s="1" t="s">
+      <c r="T32" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="S32" s="1" t="s">
+      <c r="U32" s="1" t="s">
         <v>380</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B33" s="7">
         <v>46083</v>
@@ -6101,128 +6097,128 @@
         <v>2439</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
       <c r="E33" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="H33" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="G33" s="1" t="s">
+      <c r="I33" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="K33" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="L33" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="K33" s="1" t="s">
+      <c r="P33" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="Q33" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="L33" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="M33" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="O33" s="1" t="s">
+      <c r="R33" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="P33" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="Q33" s="1" t="s">
+      <c r="S33" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="R33" s="1" t="s">
+      <c r="T33" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="S33" s="1" t="s">
+      <c r="U33" s="1" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="T33" s="1" t="s">
+      <c r="B34" s="8">
+        <v>46083</v>
+      </c>
+      <c r="C34" s="4">
+        <v>2442</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="U33" s="1" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+      <c r="E34" s="4" t="s">
         <v>393</v>
       </c>
-      <c r="B34" s="7">
-        <v>46083</v>
-      </c>
-      <c r="C34" s="1">
-        <v>2442</v>
-      </c>
-      <c r="D34" s="1" t="s">
+      <c r="F34" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I34" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="J34" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="G34" s="1" t="s">
+      <c r="K34" s="4" t="s">
         <v>396</v>
       </c>
-      <c r="H34" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="J34" s="1" t="s">
+      <c r="L34" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="M34" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="N34" s="4" t="s">
         <v>397</v>
       </c>
-      <c r="K34" s="1" t="s">
+      <c r="O34" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="L34" s="1" t="s">
+      <c r="P34" s="4" t="s">
         <v>399</v>
       </c>
-      <c r="M34" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="N34" s="1" t="s">
+      <c r="Q34" s="5" t="s">
+        <v>631</v>
+      </c>
+      <c r="R34" s="4" t="s">
         <v>400</v>
       </c>
-      <c r="O34" s="1" t="s">
+      <c r="S34" s="4" t="s">
         <v>401</v>
       </c>
-      <c r="P34" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="Q34" s="5" t="s">
-        <v>639</v>
-      </c>
-      <c r="R34" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="T34" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="U34" s="1" t="s">
-        <v>526</v>
+      <c r="T34" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="U34" s="4" t="s">
+        <v>522</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="B35" s="7">
         <v>46083</v>
@@ -6231,63 +6227,63 @@
         <v>2443</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>593</v>
+        <v>584</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>65</v>
       </c>
       <c r="I35" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="P35" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="Q35" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="R35" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="K35" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N35" s="1" t="s">
+      <c r="S35" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="O35" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="Q35" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>416</v>
-      </c>
       <c r="T35" s="1" t="s">
-        <v>594</v>
+        <v>585</v>
       </c>
       <c r="U35" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="B36" s="7">
         <v>46083</v>
@@ -6296,25 +6292,25 @@
         <v>2447</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>633</v>
+        <v>624</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>595</v>
+        <v>586</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>78</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>104</v>
@@ -6323,36 +6319,36 @@
         <v>104</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="N36" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="R36" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="O36" s="1" t="s">
+      <c r="S36" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="P36" s="1" t="s">
+      <c r="T36" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="Q36" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="R36" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="S36" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="T36" s="1" t="s">
-        <v>427</v>
-      </c>
       <c r="U36" s="1" t="s">
-        <v>596</v>
+        <v>587</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="B37" s="7">
         <v>46083</v>
@@ -6361,13 +6357,13 @@
         <v>2448</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>634</v>
+        <v>625</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>56</v>
@@ -6376,48 +6372,48 @@
         <v>197</v>
       </c>
       <c r="I37" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="O37" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="P37" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="Q37" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="L37" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="M37" s="1" t="s">
+      <c r="R37" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="S37" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="N37" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="O37" s="1" t="s">
+      <c r="T37" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="P37" s="1" t="s">
+      <c r="U37" s="1" t="s">
         <v>436</v>
-      </c>
-      <c r="Q37" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="R37" s="1" t="s">
-        <v>597</v>
-      </c>
-      <c r="S37" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="U37" s="1" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="B38" s="7">
         <v>46083</v>
@@ -6426,63 +6422,63 @@
         <v>2449</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>620</v>
+        <v>611</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="L38" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="H38" s="1" t="s">
+      <c r="M38" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="J38" s="1" t="s">
+      <c r="N38" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="K38" s="1" t="s">
+      <c r="O38" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="L38" s="1" t="s">
+      <c r="P38" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="M38" s="1" t="s">
+      <c r="Q38" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="N38" s="1" t="s">
+      <c r="R38" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="O38" s="1" t="s">
+      <c r="S38" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="P38" s="1" t="s">
+      <c r="T38" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="Q38" s="1" t="s">
+      <c r="U38" s="1" t="s">
         <v>451</v>
-      </c>
-      <c r="R38" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="S38" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="T38" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="B39" s="7">
         <v>46083</v>
@@ -6491,63 +6487,63 @@
         <v>2451</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>78</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="K39" s="1" t="s">
         <v>186</v>
       </c>
       <c r="L39" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="Q39" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="M39" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="N39" s="1" t="s">
+      <c r="R39" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="S39" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="O39" s="1" t="s">
+      <c r="T39" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="P39" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="Q39" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="R39" s="1" t="s">
-        <v>599</v>
-      </c>
-      <c r="S39" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="T39" s="1" t="s">
-        <v>464</v>
-      </c>
       <c r="U39" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="B40" s="7">
         <v>46083</v>
@@ -6556,63 +6552,63 @@
         <v>2452</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H40" s="1" t="s">
         <v>197</v>
       </c>
       <c r="I40" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="N40" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="J40" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="K40" s="1" t="s">
+      <c r="O40" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="L40" s="1" t="s">
+      <c r="P40" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="M40" s="1" t="s">
+      <c r="Q40" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="R40" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="N40" s="1" t="s">
+      <c r="S40" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="O40" s="1" t="s">
+      <c r="T40" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="P40" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="Q40" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="R40" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="S40" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="T40" s="1" t="s">
-        <v>476</v>
-      </c>
       <c r="U40" s="1" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="B41" s="7">
         <v>46083</v>
@@ -6621,63 +6617,63 @@
         <v>2504</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="I41" s="1" t="s">
         <v>478</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="J41" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>602</v>
-      </c>
-      <c r="G41" s="1" t="s">
+      <c r="K41" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="L41" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="I41" s="1" t="s">
+      <c r="M41" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="J41" s="1" t="s">
+      <c r="N41" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="O41" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="K41" s="1" t="s">
+      <c r="P41" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="L41" s="1" t="s">
+      <c r="Q41" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="M41" s="1" t="s">
+      <c r="R41" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="N41" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="O41" s="1" t="s">
+      <c r="S41" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="P41" s="1" t="s">
+      <c r="T41" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="Q41" s="1" t="s">
+      <c r="U41" s="1" t="s">
         <v>489</v>
-      </c>
-      <c r="R41" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="S41" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="T41" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="U41" s="1" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="B42" s="7">
         <v>46083</v>
@@ -6686,16 +6682,16 @@
         <v>2513</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>603</v>
+        <v>594</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>197</v>
@@ -6710,39 +6706,39 @@
         <v>104</v>
       </c>
       <c r="L42" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="M42" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="P42" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="R42" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="S42" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="T42" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="M42" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="N42" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="O42" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="P42" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="Q42" s="1" t="s">
-        <v>604</v>
-      </c>
-      <c r="R42" s="1" t="s">
-        <v>605</v>
-      </c>
-      <c r="S42" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="T42" s="1" t="s">
-        <v>501</v>
-      </c>
       <c r="U42" s="1" t="s">
-        <v>606</v>
+        <v>597</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="B43" s="7">
         <v>46083</v>
@@ -6751,22 +6747,22 @@
         <v>2545</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="H43" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>504</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>508</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>31</v>
@@ -6784,30 +6780,30 @@
         <v>31</v>
       </c>
       <c r="O43" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="S43" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="P43" s="1" t="s">
+      <c r="T43" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="Q43" s="1" t="s">
-        <v>511</v>
-      </c>
-      <c r="R43" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="S43" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="T43" s="1" t="s">
-        <v>514</v>
-      </c>
       <c r="U43" s="1" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="B44" s="7">
         <v>46083</v>
@@ -6816,13 +6812,13 @@
         <v>3682</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
@@ -6835,25 +6831,25 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
       <c r="O44" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="P44" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="R44" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="S44" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="P44" s="1" t="s">
+      <c r="T44" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="Q44" s="1" t="s">
-        <v>521</v>
-      </c>
-      <c r="R44" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="S44" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="T44" s="1" t="s">
-        <v>524</v>
-      </c>
       <c r="U44" s="1" t="s">
-        <v>607</v>
+        <v>598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>